<commit_message>
Live colour copy fix, TBD lines removed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ePhayn2UocnGVXSzVTyC3
</commit_message>
<xml_diff>
--- a/mx/BH_LiveFix_ColourCopy.xlsx
+++ b/mx/BH_LiveFix_ColourCopy.xlsx
@@ -456,7 +456,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Performance velvet upholstery in Mushroom, Terracotta, Claret, Aegean, Cream or Pewter, dense foam seat padding, stainless steel footrest, non-marking foot caps. Bar-height stools with an open curved back that runs into the arms and curved legs in one continuous upholstered line; 30.5 in seat height for bar-height counters; each rated to 330 lbs; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 38.5 in, Width 22 in, Depth 19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "30.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "38.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Performance velvet upholstery in Mushroom, Terracotta, Claret, Aegean, Cream or Pewter, dense foam seat padding, stainless steel footrest, non-marking foot caps. Bar-height stools with an open curved back that runs into the arms and curved legs in one continuous upholstered line; 30.5 in seat height for bar-height counters; each rated to 330 lbs; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 38.5 in, Width 22 in, Depth 19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "30.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "38.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -478,7 +478,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in a choice of two shades, nailhead trim, dense foam padding, sinuous spring seat support, tapered wood legs, non-marking foot caps. Upholstered dining chair with a waisted hourglass back; doubles as an accent chair for office or living room; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35.5 in, Width 24.5 in, Depth 20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in a choice of two shades, nailhead trim, dense foam padding, sinuous spring seat support, tapered wood legs, non-marking foot caps. Upholstered dining chair with a waisted hourglass back; doubles as an accent chair for office or living room; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35.5 in, Width 24.5 in, Depth 20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -500,7 +500,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Moulded acrylic in Jet (opaque gloss) or Crystal (clear), one-piece construction. Medallion-back dining armchair with oval back, curved arms and square tapering legs; 18.5 in seat height for a standard dining table; sturdy and durable; suits any room and outdoor use; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 36 in, Width 21 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "26 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Moulded acrylic in Jet (opaque gloss) or Crystal (clear), one-piece construction. Medallion-back dining armchair with oval back, curved arms and square tapering legs; 18.5 in seat height for a standard dining table; sturdy and durable; suits any room and outdoor use; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 36 in, Width 21 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "26 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -522,7 +522,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Heathered woven fabric upholstery in Heathered Stone, Heathered Dove or Heathered Cream, dense foam padding, plywood frame, solid hardwood legs and back support in Chestnut or Charcoal, fixed seat cushion, plastic floor-protecting foot pins. Armless T-back dining chair, also suited to accent use; each rated to 331 lbs; set of 2; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.5 in, Width 20.5 in, Depth 22.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Heathered woven fabric upholstery in Heathered Stone, Heathered Dove or Heathered Cream, dense foam padding, plywood frame, solid hardwood legs and back support in Chestnut or Charcoal, fixed seat cushion, plastic floor-protecting foot pins. Armless T-back dining chair, also suited to accent use; each rated to 331 lbs; set of 2; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.5 in, Width 20.5 in, Depth 22.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Performance velvet upholstery in a choice of pale shades that resists stains, dense foam over sinuous spring seat support, deep button-tufted curved back, wooden legs in a dark finish, non-marking foot caps. Tall curved-back upholstered dining chair; set of two chairs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 37.5 in, Width 18.5 in, Depth 24.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Performance velvet upholstery in a choice of pale shades that resists stains, dense foam over sinuous spring seat support, deep button-tufted curved back, wooden legs in a dark finish, non-marking foot caps. Tall curved-back upholstered dining chair; set of two chairs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 37.5 in, Width 18.5 in, Depth 24.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -566,7 +566,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven polyester fabric upholstery in Oyster or Dove, foam-padded seat, nailhead trim, tapered wooden legs in a dark finish, non-marking foot caps. Upholstered dining chair with waisted back and low flared sides, for classic or modern dining rooms; set of four chairs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 36 in, Width 22 in, Depth 25 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven polyester fabric upholstery in Oyster or Dove, foam-padded seat, nailhead trim, tapered wooden legs in a dark finish, non-marking foot caps. Upholstered dining chair with waisted back and low flared sides, for classic or modern dining rooms; set of four chairs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 36 in, Width 22 in, Depth 25 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Polyester woven fabric upholstery in a choice of colours, thick foam-padded seat and back, deep button tufting, nailhead trim, black tapered wood legs, protective foot caps. Button-tufted dining side chair with a high, gently curved back and a 20.5 in seat height; suits traditional or modern dining rooms."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 36 in, Width 21 in, Depth 25 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Polyester woven fabric upholstery in a choice of colours, thick foam-padded seat and back, deep button tufting, nailhead trim, black tapered wood legs, protective foot caps. Button-tufted dining side chair with a high, gently curved back and a 20.5 in seat height; suits traditional or modern dining rooms."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 36 in, Width 21 in, Depth 25 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -610,7 +610,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Sturdy engineered wood with a finish in Almond, Hazel or White. Two-piece home office set: a leaning, tiered ladder-frame desk with a work surface, three shelves above it and a pair of pull-out drawers, plus a wider bookcase with three open shelves over a two-door cupboard for concealed storage."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Desk: Height 71 in, Width 49 in, Depth 18.5 in; Bookcase: Height 71 in, Width 32.5 in, Depth 15.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "0.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "5.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Sturdy engineered wood with a finish in Almond, Hazel or White. Two-piece home office set: a leaning, tiered ladder-frame desk with a work surface, three shelves above it and a pair of pull-out drawers, plus a wider bookcase with three open shelves over a two-door cupboard for concealed storage."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Desk: Height 71 in, Width 49 in, Depth 18.5 in; Bookcase: Height 71 in, Width 32.5 in, Depth 15.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "0.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "5.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -632,7 +632,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood top with wood-grain veneer in Blonde, Cocoa or Hazel, bevelled edge, tapered metal pedestal stem and disc foot in White, Brass or Jet, finished to resist chips, non-marking felt floor pad. Round single-stem pedestal side table about 20 in high, level with most sofa arms; for living room, lounge corner, bedside, home office or entryway; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20 in, Width 19.5 in, Depth 19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood top with wood-grain veneer in Blonde, Cocoa or Hazel, bevelled edge, tapered metal pedestal stem and disc foot in White, Brass or Jet, finished to resist chips, non-marking felt floor pad. Round single-stem pedestal side table about 20 in high, level with most sofa arms; for living room, lounge corner, bedside, home office or entryway; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20 in, Width 19.5 in, Depth 19.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -654,7 +654,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Chestnut, slub weave upholstery in Oyster or Charcoal, foam-padded seat cushion, removable back pillow, built-in footrest rail, non-marking glides. Open-frame counter stool with arms and tapered legs; 26.5 in seat height for a kitchen counter or island; rated to 300 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 38 in, Width 22 in, Depth 22.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "26.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "31 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "2.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Chestnut, slub weave upholstery in Oyster or Charcoal, foam-padded seat cushion, removable back pillow, built-in footrest rail, non-marking glides. Open-frame counter stool with arms and tapered legs; 26.5 in seat height for a kitchen counter or island; rated to 300 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 38 in, Width 22 in, Depth 22.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "26.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "31 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "2.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft woven fabric upholstery in Mink, Charcoal or Oyster, padded seat, bentwood frame, metal foot rail, foot pins that protect floors. Counter-height barrel-back stool with a curved open back and arms that run to the floor as solid sides; 25 in seat height for a kitchen island or counter-height table; rated to 300 lbs; arrives fully assembled; sold singly."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 37 in, Width 22 in, Depth 21.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "25 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "31 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Back height above seat: ", "bold": true}, {"type": "text", "value": "12 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft woven fabric upholstery in Mink, Charcoal or Oyster, padded seat, bentwood frame, metal foot rail, foot pins that protect floors. Counter-height barrel-back stool with a curved open back and arms that run to the floor as solid sides; 25 in seat height for a kitchen island or counter-height table; rated to 300 lbs; arrives fully assembled; sold singly."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 37 in, Width 22 in, Depth 21.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "25 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "31 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Back height above seat: ", "bold": true}, {"type": "text", "value": "12 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Honey or Jet, natural woven paper cord seat, supportive back panel, X-shaped seat stretcher, non-marking floor glides. Counter-height stool for kitchen islands and counters; seat height 25.1 in; each rated to 517 lbs; set of two stools; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 38 in, Width 19 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "25.1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Width 15 in, Depth 15 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Honey or Jet, natural woven paper cord seat, supportive back panel, X-shaped seat stretcher, non-marking floor glides. Counter-height stool for kitchen islands and counters; seat height 25.1 in; each rated to 517 lbs; set of two stools; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 38 in, Width 19 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "25.1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Width 15 in, Depth 15 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frames in Chestnut finish, broad curved top rail, tapered legs with stretchers, foam-cushioned seats covered in faux leather that wipes clean, in a choice of two shades. Set of four mid-century style dining side chairs; seat height 18 in."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 29 in, Width 21.5 in, Depth 19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "15.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frames in Chestnut finish, broad curved top rail, tapered legs with stretchers, foam-cushioned seats covered in faux leather that wipes clean, in a choice of two shades. Set of four mid-century style dining side chairs; seat height 18 in."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 29 in, Width 21.5 in, Depth 19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "15.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in Pewter or Navy, deep button tufting, French piping, dense foam padding, sinuous spring seat support, carved cabriole legs in a weathered Driftwood finish, plastic foot caps. Wingback armchair for dining or for accent use in living room, bedroom, home office or entryway; 20 in seat height; each rated to 300 lbs; set of 2."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 39.5 in, Width 57 in, Depth 25.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "20.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in Pewter or Navy, deep button tufting, French piping, dense foam padding, sinuous spring seat support, carved cabriole legs in a weathered Driftwood finish, plastic foot caps. Wingback armchair for dining or for accent use in living room, bedroom, home office or entryway; 20 in seat height; each rated to 300 lbs; set of 2."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 39.5 in, Width 57 in, Depth 25.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "20.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Solid hardwood frame in Jet or Almond, woven cane backrest, bentwood seat with wood-grain veneer, non-marking foot caps. Armless cane-back dining chair, also suited to living room, office or entryway; rated to 330 lbs; single chair."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 31 in, Width 16.5 in, Depth 23.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Solid hardwood frame in Jet or Almond, woven cane backrest, bentwood seat with wood-grain veneer, non-marking foot caps. Armless cane-back dining chair, also suited to living room, office or entryway; rated to 330 lbs; single chair."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 31 in, Width 16.5 in, Depth 23.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -786,7 +786,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood frame in a choice of finishes, woven rattan seat in a natural tone. Café-style dining chair with a curved top rail, open crossed-splat back and tapered, splayed legs braced by curved hoops; 18.5 in seat height; arrives fully assembled; set of four chairs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.5 in, Width 19.5 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood frame in a choice of finishes, woven rattan seat in a natural tone. Café-style dining chair with a curved top rail, open crossed-splat back and tapered, splayed legs braced by curved hoops; 18.5 in seat height; arrives fully assembled; set of four chairs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.5 in, Width 19.5 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft hard-wearing woven fabric upholstery in Oyster or Stone, dense foam padding, bentwood seat and back shell with open back, tapered splayed stainless steel legs in Charcoal. Open-back dining side chair; rated to 331 lbs; single chair."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.5 in, Width 19.5 in, Depth 23 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft hard-wearing woven fabric upholstery in Oyster or Stone, dense foam padding, bentwood seat and back shell with open back, tapered splayed stainless steel legs in Charcoal. Open-back dining side chair; rated to 331 lbs; single chair."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.5 in, Width 19.5 in, Depth 23 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Chestnut, Driftwood, Honey or Jet, woven rattan cane back panel, foam-padded seat cushion in a pale fabric with French seam, removable cover with hidden zip, non-marking foot caps. Cane-back dining chair with a curved back; doubles as an accent chair for living room, office or entryway; each rated to 330 lbs; set of two; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 36 in, Width 18.5 in, Depth 23 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Chestnut, Driftwood, Honey or Jet, woven rattan cane back panel, foam-padded seat cushion in a pale fabric with French seam, removable cover with hidden zip, non-marking foot caps. Cane-back dining chair with a curved back; doubles as an accent chair for living room, office or entryway; each rated to 330 lbs; set of two; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 36 in, Width 18.5 in, Depth 23 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -852,7 +852,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Upholstered seat and back in a choice of colours, deep button tufting on the back, thickly padded seat cushion, dark hardwood legs with softly rounded edges, rear legs angled for balance. Upholstered dining side chair with a waisted, flared back."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 36 in, Width 18 in, Depth 24.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Upholstered seat and back in a choice of colours, deep button tufting on the back, thickly padded seat cushion, dark hardwood legs with softly rounded edges, rear legs angled for balance. Upholstered dining side chair with a waisted, flared back."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 36 in, Width 18 in, Depth 24.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -874,7 +874,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Solid hardwood frame in Blonde or Chestnut finish, Jet or Flax rope seat and back woven in a basket pattern, crossbar stretchers, non-marking foot pads. Woven dining side chair with four straight legs; 17.5 in seat height for a standard dining table; each chair rated to 331 lbs; for dining rooms, living rooms, home offices and bedrooms; assembly required; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32.5 in, Width 20 in, Depth 22.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Solid hardwood frame in Blonde or Chestnut finish, Jet or Flax rope seat and back woven in a basket pattern, crossbar stretchers, non-marking foot pads. Woven dining side chair with four straight legs; 17.5 in seat height for a standard dining table; each chair rated to 331 lbs; for dining rooms, living rooms, home offices and bedrooms; assembly required; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32.5 in, Width 20 in, Depth 22.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "1 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -896,7 +896,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Performance velvet upholstery in Mushroom, Terracotta, Claret, Aegean, Cream or Pewter, stain-resistant; dense foam padding, plywood frame, fixed contoured seat cushion, non-marking plastic glides under the base. Barrel-back dining or accent chair with an open curved back and arms in one continuous upholstered line, finishing in a sled base; 19.5 in seat height for a standard dining table; rated to 331 lbs; suits dining room, reading corner or vanity."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 27.6 in, Width 23.4 in, Depth 20.9 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "27.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height above seat: ", "bold": true}, {"type": "text", "value": "8 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Performance velvet upholstery in Mushroom, Terracotta, Claret, Aegean, Cream or Pewter, stain-resistant; dense foam padding, plywood frame, fixed contoured seat cushion, non-marking plastic glides under the base. Barrel-back dining or accent chair with an open curved back and arms in one continuous upholstered line, finishing in a sled base; 19.5 in seat height for a standard dining table; rated to 331 lbs; suits dining room, reading corner or vanity."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 27.6 in, Width 23.4 in, Depth 20.9 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "27.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height above seat: ", "bold": true}, {"type": "text", "value": "8 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -918,7 +918,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Bouclé upholstery in Charcoal, Cream, Jet or Dove, padded seat and rolled bolster backrest, solid hardwood frame in a choice of wood tones, floor-protecting foot pins. Armless dining chair on three legs with a split centre back post; for dining room, kitchen or as accent chairs; set of two; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32.99 in, Width 19.4 in, Depth 22.4 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "14.25 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "19.96 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Bouclé upholstery in Charcoal, Cream, Jet or Dove, padded seat and rolled bolster backrest, solid hardwood frame in a choice of wood tones, floor-protecting foot pins. Armless dining chair on three legs with a split centre back post; for dining room, kitchen or as accent chairs; set of two; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32.99 in, Width 19.4 in, Depth 22.4 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "14.25 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "19.96 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -940,7 +940,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in a choice of finishes, woven paper cord seat, low leg rails as a foot bar. Armless horseshoe-back dining chair with curved top rail dipping to a V at the centre, for kitchen, dining room, living room or café-style corner; seat height 17 in; rated to 331 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 28.5 in, Width 23 in, Depth 23 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "17 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "15.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in a choice of finishes, woven paper cord seat, low leg rails as a foot bar. Armless horseshoe-back dining chair with curved top rail dipping to a V at the centre, for kitchen, dining room, living room or café-style corner; seat height 17 in; rated to 331 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 28.5 in, Width 23 in, Depth 23 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "17 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "15.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft textured woven fabric upholstery in Charcoal, Fern or Dove, certified to a textile safety standard, padded seat, concealed metal frame, non-marking glides. Small sculptural accent chair with a curved barrel back, open back and three-leg form, for living room, bedroom, desk or dining use; rated to 300 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 30 in, Width 23 in, Depth 23 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "24.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft textured woven fabric upholstery in Charcoal, Fern or Dove, certified to a textile safety standard, padded seat, concealed metal frame, non-marking glides. Small sculptural accent chair with a curved barrel back, open back and three-leg form, for living room, bedroom, desk or dining use; rated to 300 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 30 in, Width 23 in, Depth 23 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "24.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Chestnut, slub weave upholstery in Oyster or Charcoal, foam-padded seat cushion, removable back pillow, non-marking glides. Open-frame dining armchair with straight arms and tapered legs; also suits a living room or a home office desk; rated to 300 lbs; comes fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 31 in, Width 22 in, Depth 22.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "21.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "24 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "2.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Chestnut, slub weave upholstery in Oyster or Charcoal, foam-padded seat cushion, removable back pillow, non-marking glides. Open-frame dining armchair with straight arms and tapered legs; also suits a living room or a home office desk; rated to 300 lbs; comes fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 31 in, Width 22 in, Depth 22.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "21.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "24 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "2.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Almond with flat arms, smooth leather sling seat and back in Caramel or Tobacco, low stretcher rails. Dining armchair for dining room, study, home office or hallway; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.1 in, Width 21.3 in, Depth 23.4 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.9 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.2 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "24 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Almond with flat arms, smooth leather sling seat and back in Caramel or Tobacco, low stretcher rails. Dining armchair for dining room, study, home office or hallway; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.1 in, Width 21.3 in, Depth 23.4 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.9 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.2 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "24 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1028,7 +1028,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft woven fabric upholstery in Charcoal or Mushroom, padded seat and curved backrest, wood legs in Hazel with solid hardwood back legs joined by a centre stretcher, non-marking foot pins. Armless curved-back dining chair for meals or working at the table; each rated to 500 lbs; set of 2; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.3 in, Width 20.8 in, Depth 22.4 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.7 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.7 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "2.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft woven fabric upholstery in Charcoal or Mushroom, padded seat and curved backrest, wood legs in Hazel with solid hardwood back legs joined by a centre stretcher, non-marking foot pins. Armless curved-back dining chair for meals or working at the table; each rated to 500 lbs; set of 2; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.3 in, Width 20.8 in, Depth 22.4 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.7 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.7 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "2.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1050,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in Moss, Truffle, Claret, Cream or Fawn, generously padded seat, bentwood frame, foot pins that protect floors. Barrel-back dining armchair with a curved back open beneath the top rail and broad squared arms that run to the floor as solid sides; 19 in seat height for a standard dining table; also suits a living room or desk; rated to 300 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 31 in, Width 23 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "25 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in Moss, Truffle, Claret, Cream or Fawn, generously padded seat, bentwood frame, foot pins that protect floors. Barrel-back dining armchair with a curved back open beneath the top rail and broad squared arms that run to the floor as solid sides; 19 in seat height for a standard dining table; also suits a living room or desk; rated to 300 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 31 in, Width 23 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "25 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1072,7 +1072,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven heathered fabric upholstery in Amber, Dove, Oyster, Charcoal, Moss or Mink over the whole chair, arms and legs included, elastic webbing seat support, thick dense foam seat cushion, bracket system that holds the backrest secure, floor glides. Upholstered dining armchair with squared arms, a low back and angled legs; 20.2 in seat height for a standard dining table; rated to 500 lbs; suits dining rooms, bedrooms, home offices and living rooms; assembly required; single chair."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.5 in, Width 24.4 in, Depth 26.6 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20.2 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "19.3 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "5.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven heathered fabric upholstery in Amber, Dove, Oyster, Charcoal, Moss or Mink over the whole chair, arms and legs included, elastic webbing seat support, thick dense foam seat cushion, bracket system that holds the backrest secure, floor glides. Upholstered dining armchair with squared arms, a low back and angled legs; 20.2 in seat height for a standard dining table; rated to 500 lbs; suits dining rooms, bedrooms, home offices and living rooms; assembly required; single chair."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.5 in, Width 24.4 in, Depth 26.6 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20.2 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "19.3 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "5.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1094,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame with reinforced stretchers, dense foam padding, removable floor-length slipcover in a textured slub-weave polyester in a choice of plain shades and windowpane checks (spot clean). Tall, gently curved back parsons-style slipcovered dining side chair for the dining room, a breakfast nook or occasional seating; each rated to 300 lbs; set of two; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 37 in, Width 19.5 in, Depth 24.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Back height above seat: ", "bold": true}, {"type": "text", "value": "17 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "5.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame with reinforced stretchers, dense foam padding, removable floor-length slipcover in a textured slub-weave polyester in a choice of plain shades and windowpane checks (spot clean). Tall, gently curved back parsons-style slipcovered dining side chair for the dining room, a breakfast nook or occasional seating; each rated to 300 lbs; set of two; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 37 in, Width 19.5 in, Depth 24.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Back height above seat: ", "bold": true}, {"type": "text", "value": "17 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "5.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1116,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood frame in a choice of finishes with low stretchers between the legs, seat and back panel woven from natural twisted paper cord, plastic foot glides. Square-framed woven-seat dining side chair, also suited to use as an accent chair; each rated to 330 lbs; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.6 in, Width 20.1 in, Depth 24 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "17.9 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18.9 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "2.8 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood frame in a choice of finishes with low stretchers between the legs, seat and back panel woven from natural twisted paper cord, plastic foot glides. Square-framed woven-seat dining side chair, also suited to use as an accent chair; each rated to 330 lbs; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.6 in, Width 20.1 in, Depth 24 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "17.9 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18.9 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "2.8 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1138,7 +1138,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood case with wood-grain laminate in a choice of finishes, edge trim, tempered glass doors, tapered wood legs, soft-close hinges, brass-toned metal ring pulls, full-glide drawers, non-marking foot pads. Tall arch-topped display cabinet with an open arched shelf, then a fixed shelf, two adjustable shelves and drawers behind two glazed doors; rated loads: arched shelf 88 lb, adjustable shelves 70 lb, fixed shelf 62 lb, drawers 22 lb; for a living room, dining room or hallway; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 71 in, Width 31 in, Depth 16.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Shelf: ", "bold": true}, {"type": "text", "value": "Height 9 in, Width 30.5 in, Depth 13.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood case with wood-grain laminate in a choice of finishes, edge trim, tempered glass doors, tapered wood legs, soft-close hinges, brass-toned metal ring pulls, full-glide drawers, non-marking foot pads. Tall arch-topped display cabinet with an open arched shelf, then a fixed shelf, two adjustable shelves and drawers behind two glazed doors; rated loads: arched shelf 88 lb, adjustable shelves 70 lb, fixed shelf 62 lb, drawers 22 lb; for a living room, dining room or hallway; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 71 in, Width 31 in, Depth 16.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Shelf: ", "bold": true}, {"type": "text", "value": "Height 9 in, Width 30.5 in, Depth 13.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1160,7 +1160,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood with a wood-grain laminate finish in Honey or Hazel, woven synthetic rattan door panels, two full-height doors with soft-close hinges, two adjustable shelves, non-marking adjustable levelers. Tall arched linen and storage cabinet for hallway, office or living room; assembly required; weight capacity not stated."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 78.7 in, Width 45.9 in, Depth 15.6 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Shelf: ", "bold": true}, {"type": "text", "value": "Height 20.8 in, Width 42.8 in, Depth 13.2 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood with a wood-grain laminate finish in Honey or Hazel, woven synthetic rattan door panels, two full-height doors with soft-close hinges, two adjustable shelves, non-marking adjustable levelers. Tall arched linen and storage cabinet for hallway, office or living room; assembly required; weight capacity not stated."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 78.7 in, Width 45.9 in, Depth 15.6 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Shelf: ", "bold": true}, {"type": "text", "value": "Height 20.8 in, Width 42.8 in, Depth 13.2 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1182,7 +1182,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood in Chestnut or Almond finish, carved scalloped door fronts, three doors with finger pulls, interior shelving, covered cable holes in the back, round bun feet fitted with levelers. Low three-door media cabinet with a deeply ribbed vertical front; top suits televisions up to 60 in; rated to 154 lbs concentrated load; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 17.5 in, Width 54 in, Depth 16 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood in Chestnut or Almond finish, carved scalloped door fronts, three doors with finger pulls, interior shelving, covered cable holes in the back, round bun feet fitted with levelers. Low three-door media cabinet with a deeply ribbed vertical front; top suits televisions up to 60 in; rated to 154 lbs concentrated load; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 17.5 in, Width 54 in, Depth 16 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood with wood-grain laminate finish in Jet or Almond, four push-to-open doors with raised grid panels, adjustable interior shelves (three positions), four tapered legs with a central levelling leg, non-marking foot pads. Sideboard for dining buffet, media stand, hall or office storage; top rated to 308 lbs, interior shelves to 83 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32.2 in, Width 62.1 in, Depth 17.8 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside: ", "bold": true}, {"type": "text", "value": "6.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood with wood-grain laminate finish in Jet or Almond, four push-to-open doors with raised grid panels, adjustable interior shelves (three positions), four tapered legs with a central levelling leg, non-marking foot pads. Sideboard for dining buffet, media stand, hall or office storage; top rated to 308 lbs, interior shelves to 83 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32.2 in, Width 62.1 in, Depth 17.8 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside: ", "bold": true}, {"type": "text", "value": "6.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood and engineered wood construction in Oyster, Jet or Chestnut, carved basketweave relief across both doors, adjustable interior shelves, magnetic door catches, rear cable holes for TV and media wiring, low plinth feet. Wide, low two-door sideboard that works as a buffet, credenza or media cabinet beneath a wall-mounted TV; for dining rooms, living rooms, halls and entries; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33 in, Width 71 in, Depth 18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside: ", "bold": true}, {"type": "text", "value": "4.3 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Height 16.9 in, Width 33.9 in, Depth 15.9 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood and engineered wood construction in Oyster, Jet or Chestnut, carved basketweave relief across both doors, adjustable interior shelves, magnetic door catches, rear cable holes for TV and media wiring, low plinth feet. Wide, low two-door sideboard that works as a buffet, credenza or media cabinet beneath a wall-mounted TV; for dining rooms, living rooms, halls and entries; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33 in, Width 71 in, Depth 18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside: ", "bold": true}, {"type": "text", "value": "4.3 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Height 16.9 in, Width 33.9 in, Depth 15.9 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Finish in Chestnut, Oyster or Jet, stepped-profile frame, fluted end panels, square block pulls, two interior shelves each adjustable to five heights, four cable openings in the back panel. Four-door sideboard with two compartments, for dining room storage, a bar or a media cabinet below a wall-hung television; top rated to 110 lbs, each shelf 44 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 31.8 in, Width 70.2 in, Depth 17.8 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Height 25.3 in, Width 29.4 in, Depth 14.2 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Finish in Chestnut, Oyster or Jet, stepped-profile frame, fluted end panels, square block pulls, two interior shelves each adjustable to five heights, four cable openings in the back panel. Four-door sideboard with two compartments, for dining room storage, a bar or a media cabinet below a wall-hung television; top rated to 110 lbs, each shelf 44 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 31.8 in, Width 70.2 in, Depth 17.8 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Height 25.3 in, Width 29.4 in, Depth 14.2 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1270,7 +1270,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Sturdy engineered wood with a finish in Almond, Hazel or White. Three-piece home office set: a leaning, tiered ladder-frame desk with a work surface, three shelves above it and a pair of pull-out drawers, plus two wider bookcases, each with three open shelves over a two-door cupboard for concealed storage."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 71 in, Width 114 in, Depth 18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "0.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "4.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Sturdy engineered wood with a finish in Almond, Hazel or White. Three-piece home office set: a leaning, tiered ladder-frame desk with a work surface, three shelves above it and a pair of pull-out drawers, plus two wider bookcases, each with three open shelves over a two-door cupboard for concealed storage."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 71 in, Width 114 in, Depth 18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "0.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "4.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1292,7 +1292,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood frame and four open wood shelves in Blonde, Jet or Chestnut, matching arched frames front and back, open back and sides, non-marking glides. Tall, wide open bookcase about 6 ft high, for books, collected pieces and display; shelves hold up to 220 lbs in all; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 72.1 in, Width 36 in, Depth 14.1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Shelf: ", "bold": true}, {"type": "text", "value": "Height 1.2 in, Width 36 in, Depth 14.1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood frame and four open wood shelves in Blonde, Jet or Chestnut, matching arched frames front and back, open back and sides, non-marking glides. Tall, wide open bookcase about 6 ft high, for books, collected pieces and display; shelves hold up to 220 lbs in all; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 72.1 in, Width 36 in, Depth 14.1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Shelf: ", "bold": true}, {"type": "text", "value": "Height 1.2 in, Width 36 in, Depth 14.1 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Real burl wood veneer in Almond or Honey over an engineered wood core, adjustable leveling feet with non-marking pads. Round drum side table with veneer wrapped across the top and sides; each figure is unique; rated to 298 lbs; no assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20.5 in, Width 16 in, Depth 16 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Real burl wood veneer in Almond or Honey over an engineered wood core, adjustable leveling feet with non-marking pads. Round drum side table with veneer wrapped across the top and sides; each figure is unique; rated to 298 lbs; no assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20.5 in, Width 16 in, Depth 16 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1336,7 +1336,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Natural marble sphere base, iron rod and round iron top in a White, Jet or Brass finish, non-marking pad. Slim drinks side table for beside an armchair or sofa, or as a plant stand; rated to 99 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20 in, Width 14 in, Depth 14 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Natural marble sphere base, iron rod and round iron top in a White, Jet or Brass finish, non-marking pad. Slim drinks side table for beside an armchair or sofa, or as a plant stand; rated to 99 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20 in, Width 14 in, Depth 14 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood with a concrete finish in Cream or Jet, felt floor pads. Round side table with a deep, bowl-edged top on a three-lobed clover pedestal; compact enough for small spaces, beside a sofa or bed or in a hall; rated to 198 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 21.8 in, Width 17.7 in, Depth 17.7 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood with a concrete finish in Cream or Jet, felt floor pads. Round side table with a deep, bowl-edged top on a three-lobed clover pedestal; compact enough for small spaces, beside a sofa or bed or in a hall; rated to 198 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 21.8 in, Width 17.7 in, Depth 17.7 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1380,7 +1380,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Sintered stone top in White, waterproof, resists stains, scratches and heat, safe with household cleaners, tapered metal pedestal stem and disc foot in Jet or Brass. Round single-stem pedestal side table about 20 in high, level with most sofa arms; for living room, lounge corner, bedside, home office or entryway."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20.5 in, Width 19.5 in, Depth 19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Sintered stone top in White, waterproof, resists stains, scratches and heat, safe with household cleaners, tapered metal pedestal stem and disc foot in Jet or Brass. Round single-stem pedestal side table about 20 in high, level with most sofa arms; for living room, lounge corner, bedside, home office or entryway."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20.5 in, Width 19.5 in, Depth 19.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1402,7 +1402,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Laminated engineered wood with a wood-grain finish in Almond or Hazel, woven synthetic rattan drawer fronts, seven drawers (four upper, three lower), long open lower shelf, non-marking foot pads. Narrow console table for entry, hallway or behind a sofa; rated to 194 lbs distributed, 11 lbs per drawer, 154 lbs on the lower shelf."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.9 in, Width 62.6 in, Depth 15.4 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Drawer interior: ", "bold": true}, {"type": "text", "value": "Height 3.9 in, Width 16.7 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Laminated engineered wood with a wood-grain finish in Almond or Hazel, woven synthetic rattan drawer fronts, seven drawers (four upper, three lower), long open lower shelf, non-marking foot pads. Narrow console table for entry, hallway or behind a sofa; rated to 194 lbs distributed, 11 lbs per drawer, 154 lbs on the lower shelf."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.9 in, Width 62.6 in, Depth 15.4 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Drawer interior: ", "bold": true}, {"type": "text", "value": "Height 3.9 in, Width 16.7 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1424,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Real burl wood veneer in Almond or Honey over an engineered wood core, adjustable leveling feet with non-marking pads. Low square block coffee table with veneer wrapped across the top and sides; each figure is unique; rated to 440 lbs; no assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 16 in, Width 36 in, Depth 36 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Real burl wood veneer in Almond or Honey over an engineered wood core, adjustable leveling feet with non-marking pads. Low square block coffee table with veneer wrapped across the top and sides; each figure is unique; rated to 440 lbs; no assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 16 in, Width 36 in, Depth 36 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1556,7 +1556,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Moulded acrylic in Cobalt, Blush or Pewter tint (translucent), one-piece construction. Medallion-back dining armchair with oval back, curved arms and square tapering legs; 18.5 in seat height for a standard dining table; sturdy and durable; suits any room and outdoor use; sold singly."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 36 in, Width 22 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "26.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Moulded acrylic in Cobalt, Blush or Pewter tint (translucent), one-piece construction. Medallion-back dining armchair with oval back, curved arms and square tapering legs; 18.5 in seat height for a standard dining table; sturdy and durable; suits any room and outdoor use; sold singly."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 36 in, Width 22 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "26.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Performance velvet upholstery in Cream, Bottle Green, Pewter or Old Rose, stain-resistant, button-tufted back and seat, thickly padded 4.5 in seat cushion, flat-bar stainless steel sled base and back frame in a Brass finish. Square-backed armless dining chair; 18.5 in seat height for a standard dining table; rated to 331 lbs; arrives ready to use, no assembly needed."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35.5 in, Width 19 in, Depth 25.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Performance velvet upholstery in Cream, Bottle Green, Pewter or Old Rose, stain-resistant, button-tufted back and seat, thickly padded 4.5 in seat cushion, flat-bar stainless steel sled base and back frame in a Brass finish. Square-backed armless dining chair; 18.5 in seat height for a standard dining table; rated to 331 lbs; arrives ready to use, no assembly needed."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35.5 in, Width 19 in, Depth 25.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "19 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1600,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Moulded acrylic in Pewter or Citron tint (translucent), one-piece construction. Armless medallion-back dining chair with oval back and square tapering legs; 18.5 in seat height for a standard dining table; sturdy and durable; suits any room and outdoor use; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35.5 in, Width 15 in, Depth 19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Moulded acrylic in Pewter or Citron tint (translucent), one-piece construction. Armless medallion-back dining chair with oval back and square tapering legs; 18.5 in seat height for a standard dining table; sturdy and durable; suits any room and outdoor use; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35.5 in, Width 15 in, Depth 19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1622,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid wood frame in Jet or Honey, woven faux cane back panel in a dark or natural tone, dense foam seat upholstered in heathered fabric in Heathered Cream or Heathered Flax, non-marking foot glides. Tall-backed dining side chair with a squared frame and square legs, also at home as an accent chair; rated to 551 lbs; set of two; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 39 in, Width 19.7 in, Depth 23.2 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.425 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.915 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid wood frame in Jet or Honey, woven faux cane back panel in a dark or natural tone, dense foam seat upholstered in heathered fabric in Heathered Cream or Heathered Flax, non-marking foot glides. Tall-backed dining side chair with a squared frame and square legs, also at home as an accent chair; rated to 551 lbs; set of two; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 39 in, Width 19.7 in, Depth 23.2 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.425 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.915 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1644,7 +1644,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in Pewter or Chambray, dense foam padding, wood and plywood frame, splayed brushed Brass-tone stainless steel legs with non-marking caps, Brass-tone pull on the outer back for drawing the chair out. Scoop-back upholstered dining armchair with low sloping arms; outer back finished in vertical pleats; also suits a desk, vanity, bedroom, living room or entryway; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34 in, Width 50 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in Pewter or Chambray, dense foam padding, wood and plywood frame, splayed brushed Brass-tone stainless steel legs with non-marking caps, Brass-tone pull on the outer back for drawing the chair out. Scoop-back upholstered dining armchair with low sloping arms; outer back finished in vertical pleats; also suits a desk, vanity, bedroom, living room or entryway; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34 in, Width 50 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "19 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1666,7 +1666,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven fabric upholstery in a choice of shades, dense foam padding, solid wood and engineered wood frame, wooden legs in a dark finish, non-marking foot glides, silver-toned nailhead trim. Tall flared-back Parsons-style dining chair for the dining table, a home office desk, a hall or a living room; rated to 500 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 40 in, Width 19.5 in, Depth 23.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "6 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven fabric upholstery in a choice of shades, dense foam padding, solid wood and engineered wood frame, wooden legs in a dark finish, non-marking foot glides, silver-toned nailhead trim. Tall flared-back Parsons-style dining chair for the dining table, a home office desk, a hall or a living room; rated to 500 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 40 in, Width 19.5 in, Depth 23.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "6 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1688,7 +1688,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Solid kiln-dried hardwood with wood veneer, in Jet, Honey or Cocoa, two tempered glass doors with arched panes, soft-close doors, magnetic push-to-open catch, four fixed shelves plus a concealed lower shelf. Tall arched display cabinet that serves as china cabinet, curio or glazed bookcase in dining rooms, living rooms and home libraries; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 79 in, Width 40 in, Depth 16 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Solid kiln-dried hardwood with wood veneer, in Jet, Honey or Cocoa, two tempered glass doors with arched panes, soft-close doors, magnetic push-to-open catch, four fixed shelves plus a concealed lower shelf. Tall arched display cabinet that serves as china cabinet, curio or glazed bookcase in dining rooms, living rooms and home libraries; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 79 in, Width 40 in, Depth 16 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1710,7 +1710,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Sturdy engineered wood in a choice of finishes. Set of two leaning, tiered ladder-frame bookcases, one narrow and one wide, each with three open shelves over a cupboard for concealed storage (one door on the narrow, two on the wide)."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Narrow bookcase: Height 71 in, Width 20.5 in, Depth 15 in; Wide bookcase: Height 71 in, Width 32.5 in, Depth 15.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "5.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "0.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Sturdy engineered wood in a choice of finishes. Set of two leaning, tiered ladder-frame bookcases, one narrow and one wide, each with three open shelves over a cupboard for concealed storage (one door on the narrow, two on the wide)."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Narrow bookcase: Height 71 in, Width 20.5 in, Depth 15 in; Wide bookcase: Height 71 in, Width 32.5 in, Depth 15.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "5.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "0.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood top in White high-gloss finish, bevelled edge, tapered metal pedestal stem and disc foot in White, Brass or Jet, with a finish that resists chips, non-marking felt floor pad. Round single-stem pedestal side table about 20 in high, level with most sofa arms; for living room, lounge corner, bedside, home office or entryway; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20 in, Width 19.5 in, Depth 19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood top in White high-gloss finish, bevelled edge, tapered metal pedestal stem and disc foot in White, Brass or Jet, with a finish that resists chips, non-marking felt floor pad. Round single-stem pedestal side table about 20 in high, level with most sofa arms; for living room, lounge corner, bedside, home office or entryway; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20 in, Width 19.5 in, Depth 19.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1754,7 +1754,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft, durable woven polyester upholstery in a choice of shades, button-tufted padded back and seat, thickly padded 4.5 in seat cushions, flat-bar stainless steel sled bases with footrest bars and back frames in a Brass finish. Pair of counter-height stools with low square backs; 26.5 in seat height; each stool rated to 331 lbs; set of two; arrives ready to use, no assembly needed."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 38 in, Width 38 in, Depth 23 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "26.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "4.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft, durable woven polyester upholstery in a choice of shades, button-tufted padded back and seat, thickly padded 4.5 in seat cushions, flat-bar stainless steel sled bases with footrest bars and back frames in a Brass finish. Pair of counter-height stools with low square backs; 26.5 in seat height; each stool rated to 331 lbs; set of two; arrives ready to use, no assembly needed."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 38 in, Width 38 in, Depth 23 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "26.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "4.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in Moss, Claret, Cream, Truffle or Fawn, padded seat, bentwood frame, metal foot rail, foot pins that protect floors. Bar-height barrel-back stool with a curved open back and arms that run to the floor as solid sides; 28.5 in seat height for a standard home bar; rated to 300 lbs; arrives fully assembled; sold singly."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 41 in, Width 22 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "28.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "35 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Back height above seat: ", "bold": true}, {"type": "text", "value": "12 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in Moss, Claret, Cream, Truffle or Fawn, padded seat, bentwood frame, metal foot rail, foot pins that protect floors. Bar-height barrel-back stool with a curved open back and arms that run to the floor as solid sides; 28.5 in seat height for a standard home bar; rated to 300 lbs; arrives fully assembled; sold singly."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 41 in, Width 22 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "28.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "35 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Back height above seat: ", "bold": true}, {"type": "text", "value": "12 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1798,7 +1798,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Chestnut finish, broad curved top rail, tapered legs with stretchers, foam-cushioned seat covered in faux leather in a choice of shades that wipes clean. Mid-century style dining side chair; seat height 17.5 in."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 29 in, Width 19 in, Depth 21.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Chestnut finish, broad curved top rail, tapered legs with stretchers, foam-cushioned seat covered in faux leather in a choice of shades that wipes clean. Mid-century style dining side chair; seat height 17.5 in."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 29 in, Width 19 in, Depth 21.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1820,7 +1820,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood frame in a choice of finishes, woven rattan seat in a natural tone. Café-style dining chair with a curved top rail, open crossed-splat back and tapered, splayed legs braced by curved hoops; 18.5 in seat height; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.5 in, Width 19.5 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood frame in a choice of finishes, woven rattan seat in a natural tone. Café-style dining chair with a curved top rail, open crossed-splat back and tapered, splayed legs braced by curved hoops; 18.5 in seat height; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.5 in, Width 19.5 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1842,7 +1842,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft hard-wearing woven fabric upholstery in Oyster or Stone, dense foam padding, bentwood seat and back shell with open back, tapered splayed stainless steel legs in Charcoal. Open-back dining side chair; each rated to 331 lbs; set of 2."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.5 in, Width 39 in, Depth 23 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft hard-wearing woven fabric upholstery in Oyster or Stone, dense foam padding, bentwood seat and back shell with open back, tapered splayed stainless steel legs in Charcoal. Open-back dining side chair; each rated to 331 lbs; set of 2."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.5 in, Width 39 in, Depth 23 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven rattan cane seat and back, hardwood frame in Jet or Driftwood, rounded edges, ring stretcher, non-marking foot caps. Armless cane-back dining side chair, also an accent or desk chair; 18.5 in seat height; rated to 330 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32 in, Width 17.5 in, Depth 20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven rattan cane seat and back, hardwood frame in Jet or Driftwood, rounded edges, ring stretcher, non-marking foot caps. Armless cane-back dining side chair, also an accent or desk chair; 18.5 in seat height; rated to 330 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32 in, Width 17.5 in, Depth 20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1886,7 +1886,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven fabric upholstery in Oyster, Bark or Pewter, dense foam padding, solid wood frame, dark-finished wooden legs, non-marking foot glides, silver-toned nailhead trim. Tall flared-back Parsons-style dining chair; set of four chairs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 40 in, Width 19.5 in, Depth 23.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven fabric upholstery in Oyster, Bark or Pewter, dense foam padding, solid wood frame, dark-finished wooden legs, non-marking foot glides, silver-toned nailhead trim. Tall flared-back Parsons-style dining chair; set of four chairs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 40 in, Width 19.5 in, Depth 23.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1908,7 +1908,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Durable woven polyester upholstery in a choice of shades, dense foam padding, tapered stainless steel legs in a matte Jet finish. Pair of armless dining chairs with tall curved backs and defined seat cushions; 19 in seat height; each chair rated to 300 lbs; works as dining or accent seating; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.5 in, Width 19 in, Depth 23 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Durable woven polyester upholstery in a choice of shades, dense foam padding, tapered stainless steel legs in a matte Jet finish. Pair of armless dining chairs with tall curved backs and defined seat cushions; 19 in seat height; each chair rated to 300 lbs; works as dining or accent seating; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.5 in, Width 19 in, Depth 23 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1930,7 +1930,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame, performance velvet upholstery that resists stains, dense foam over sinuous spring seat support, deep button tufting on the inside back, non-marking floor glides. Tall winged dining chairs with curved backs; 20 in seat height; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 38.5 in, Width 21 in, Depth 26.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame, performance velvet upholstery that resists stains, dense foam over sinuous spring seat support, deep button tufting on the inside back, non-marking floor glides. Tall winged dining chairs with curved backs; 20 in seat height; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 38.5 in, Width 21 in, Depth 26.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1952,7 +1952,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven polyester fabric upholstery in a choice of shades, nailhead trim, dense foam padding, webbing and zigzag spring seat support that resists sagging, tapered wood legs, non-marking foot caps. Upholstered dining chair with a waisted hourglass back; for dining table, desk or bedroom; sold singly."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 36 in, Width 25 in, Depth 23 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven polyester fabric upholstery in a choice of shades, nailhead trim, dense foam padding, webbing and zigzag spring seat support that resists sagging, tapered wood legs, non-marking foot caps. Upholstered dining chair with a waisted hourglass back; for dining table, desk or bedroom; sold singly."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 36 in, Width 25 in, Depth 23 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1974,7 +1974,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Performance velvet upholstery, stain-resistant, in Cream or Truffle, dense foam over plywood seat and back, fixed seat cushion, wood legs in Hazel, non-marking foot pins. Barrel-back upholstered dining chairs with curved open back, also suit use as small accent chairs; set of two; rated to 331 lbs each; easy assembly."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 28.7 in, Width 25.2 in, Depth 22.1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "28.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Performance velvet upholstery, stain-resistant, in Cream or Truffle, dense foam over plywood seat and back, fixed seat cushion, wood legs in Hazel, non-marking foot pins. Barrel-back upholstered dining chairs with curved open back, also suit use as small accent chairs; set of two; rated to 331 lbs each; easy assembly."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 28.7 in, Width 25.2 in, Depth 22.1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "28.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood frame in Jet or Honey, woven rattan cane back panel, dense foam seat upholstered in heathered fabric in Pewter, non-marking floor glides. Armless cane-back dining side chair with slim legs; also suits a living room or home office; rated to 330 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.5 in, Width 19.1 in, Depth 20.9 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood frame in Jet or Honey, woven rattan cane back panel, dense foam seat upholstered in heathered fabric in Pewter, non-marking floor glides. Armless cane-back dining side chair with slim legs; also suits a living room or home office; rated to 330 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.5 in, Width 19.1 in, Depth 20.9 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2018,7 +2018,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood frame in a choice of finishes with tapered arms and splayed A-frame legs, woven cane backrest, padded faux leather seat cushion in Charcoal or Stone. Dining armchair for dining or kitchen table, or as a living room accent chair; each rated to 507 lbs; set of 2; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32.5 in, Width 20.4 in, Depth 22.4 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "25.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood frame in a choice of finishes with tapered arms and splayed A-frame legs, woven cane backrest, padded faux leather seat cushion in Charcoal or Stone. Dining armchair for dining or kitchen table, or as a living room accent chair; each rated to 507 lbs; set of 2; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32.5 in, Width 20.4 in, Depth 22.4 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "25.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven polyester upholstery in a choice of shades, dense foam padding throughout, tapered wood legs in a Charcoal finish. Armless upholstered dining side chair with a tall curved back that flares at the shoulders and a defined seat cushion; 19 in seat height for a standard dining table; also suits a desk or dressing table."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34 in, Width 19 in, Depth 24 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven polyester upholstery in a choice of shades, dense foam padding throughout, tapered wood legs in a Charcoal finish. Armless upholstered dining side chair with a tall curved back that flares at the shoulders and a defined seat cushion; 19 in seat height for a standard dining table; also suits a desk or dressing table."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34 in, Width 19 in, Depth 24 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2062,7 +2062,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Textured woven fabric upholstery in Stone, Cream, Fern or Navy, certified free of harmful substances, padded seat and rounded back, polished Chrome-finish metal frame forming supportive arms and a sled base, adjustable non-marking glides. Compact barrel-back accent chair, also suited to desk, vanity or dining use; rated to 300 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 30.5 in, Width 21.5 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "27 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Textured woven fabric upholstery in Stone, Cream, Fern or Navy, certified free of harmful substances, padded seat and rounded back, polished Chrome-finish metal frame forming supportive arms and a sled base, adjustable non-marking glides. Compact barrel-back accent chair, also suited to desk, vanity or dining use; rated to 300 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 30.5 in, Width 21.5 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "27 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2084,7 +2084,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame, tapered legs and bracing stretchers in a Chestnut, Jet or Honey finish, woven paper cord seat that is soft, static-free and hard-wearing. Spindle-back dining side chair with a deep curved top rail, for dining room, kitchen or living area; seat height 18.5 in; rated to 286 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 31.5 in, Width 22.5 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "15.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame, tapered legs and bracing stretchers in a Chestnut, Jet or Honey finish, woven paper cord seat that is soft, static-free and hard-wearing. Spindle-back dining side chair with a deep curved top rail, for dining room, kitchen or living area; seat height 18.5 in; rated to 286 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 31.5 in, Width 22.5 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "15.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2106,7 +2106,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in a choice of wood tones, smooth leather sling seat and back in Caramel or Tobacco, low stretcher rails. Armless dining side chair for dining room, study, home office or hallway; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.1 in, Width 21.7 in, Depth 23.2 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.9 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in a choice of wood tones, smooth leather sling seat and back in Caramel or Tobacco, low stretcher rails. Armless dining side chair for dining room, study, home office or hallway; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.1 in, Width 21.7 in, Depth 23.2 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.9 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft fabric upholstery in Mushroom or Charcoal, padded curved open backrest and round seat cushion, wood frame and cylindrical legs in Hazel, non-marking foot pins. Small curved-back accent chairs, also usable at a dining table, set of two; rated to 500 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 30.4 in, Width 23.9 in, Depth 22.8 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.7 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "21.1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "2.6 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft fabric upholstery in Mushroom or Charcoal, padded curved open backrest and round seat cushion, wood frame and cylindrical legs in Hazel, non-marking foot pins. Small curved-back accent chairs, also usable at a dining table, set of two; rated to 500 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 30.4 in, Width 23.9 in, Depth 22.8 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.7 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "21.1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "2.6 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2150,7 +2150,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Slub weave fabric upholstery in Oyster, Mink or Charcoal, generously padded seat, bentwood frame, foot pins that protect floors. Barrel-back dining armchair with a curved back open beneath the top rail and broad squared arms that run to the floor as solid sides; 19 in seat height for a standard dining table; also suits a living room or desk; rated to 300 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 31 in, Width 23 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "25 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Slub weave fabric upholstery in Oyster, Mink or Charcoal, generously padded seat, bentwood frame, foot pins that protect floors. Barrel-back dining armchair with a curved back open beneath the top rail and broad squared arms that run to the floor as solid sides; 19 in seat height for a standard dining table; also suits a living room or desk; rated to 300 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 31 in, Width 23 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "25 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in Claret, Mushroom or Cream over the whole chair, arms and legs included, elastic webbing seat support, thick dense foam seat cushion, bracket system that holds the backrest secure, floor glides. Upholstered dining armchair with squared arms, a low back and angled legs; 20.2 in seat height for a standard dining table; rated to 500 lbs; suits dining rooms, bedrooms, home offices and living rooms; assembly required; single chair."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.5 in, Width 24.4 in, Depth 26.6 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20.2 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "19.3 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "5.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in Claret, Mushroom or Cream over the whole chair, arms and legs included, elastic webbing seat support, thick dense foam seat cushion, bracket system that holds the backrest secure, floor glides. Upholstered dining armchair with squared arms, a low back and angled legs; 20.2 in seat height for a standard dining table; rated to 500 lbs; suits dining rooms, bedrooms, home offices and living rooms; assembly required; single chair."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.5 in, Width 24.4 in, Depth 26.6 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20.2 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "19.3 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "5.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2194,7 +2194,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Linen-blend fabric upholstery in Oat Ticking Stripe, Chambray Ticking Stripe, Cream, Mushroom or Olive, dense foam cushioning with a supportive back, scalloped back flowing into gently flared rounded arms, concealed swivel base that turns 360 degrees, cover tailored down to the floor. Swivel dining chair for dining tables, breakfast nooks and eat-in kitchens; seat height 19.5 in; rated to 300 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34 in, Width 24 in, Depth 27.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "21.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "26 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Back height above seat: ", "bold": true}, {"type": "text", "value": "14.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Linen-blend fabric upholstery in Oat Ticking Stripe, Chambray Ticking Stripe, Cream, Mushroom or Olive, dense foam cushioning with a supportive back, scalloped back flowing into gently flared rounded arms, concealed swivel base that turns 360 degrees, cover tailored down to the floor. Swivel dining chair for dining tables, breakfast nooks and eat-in kitchens; seat height 19.5 in; rated to 300 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34 in, Width 24 in, Depth 27.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "21.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "26 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Back height above seat: ", "bold": true}, {"type": "text", "value": "14.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2216,7 +2216,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Honey or Hazel, open-weave cord seat and curved backrest in Flax, splayed legs with stretchers. Armless woven dining side chairs for the dining room or a kitchen nook, set of two; each rated to 517 lbs; arrive fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35 in, Width 19 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.3 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.9 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Width 16.4 in, Depth 16.3 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Honey or Hazel, open-weave cord seat and curved backrest in Flax, splayed legs with stretchers. Armless woven dining side chairs for the dining room or a kitchen nook, set of two; each rated to 517 lbs; arrive fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35 in, Width 19 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.3 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.9 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Width 16.4 in, Depth 16.3 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2238,7 +2238,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood-grain laminate case in Jet, Cream, Almond or Cocoa, edge trim, tempered glass doors, tapered wood legs, soft-close hinges, brass-toned metal ring pulls, full-glide drawers, non-marking foot pads. Tall arch-topped display cabinet with an open arched shelf, then a fixed shelf, two adjustable shelves and drawers behind two glazed doors; rated loads: arched shelf 88 lb, adjustable shelves 70 lb, fixed shelf 62 lb, drawers 22 lb; for a living room, dining room or hallway; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 74.1 in, Width 39.37 in, Depth 16.61 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Height 46.89 in, Width 37.56 in, Depth 15.04 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood-grain laminate case in Jet, Cream, Almond or Cocoa, edge trim, tempered glass doors, tapered wood legs, soft-close hinges, brass-toned metal ring pulls, full-glide drawers, non-marking foot pads. Tall arch-topped display cabinet with an open arched shelf, then a fixed shelf, two adjustable shelves and drawers behind two glazed doors; rated loads: arched shelf 88 lb, adjustable shelves 70 lb, fixed shelf 62 lb, drawers 22 lb; for a living room, dining room or hallway; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 74.1 in, Width 39.37 in, Depth 16.61 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Height 46.89 in, Width 37.56 in, Depth 15.04 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2260,7 +2260,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood-grain finish in Oyster or Jet, two full-height soft-close doors with long vertical pulls, two adjustable shelves and one fixed shelf, rounded feet on non-marking glides. Tall arch-topped storage cabinet for pantry, linen or household storage in kitchen, dining or living room; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 79.1 in, Width 38.2 in, Depth 15.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Shelf: ", "bold": true}, {"type": "text", "value": "Height 39.3 in, Width 34.9 in, Depth 13 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood-grain finish in Oyster or Jet, two full-height soft-close doors with long vertical pulls, two adjustable shelves and one fixed shelf, rounded feet on non-marking glides. Tall arch-topped storage cabinet for pantry, linen or household storage in kitchen, dining or living room; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 79.1 in, Width 38.2 in, Depth 15.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Shelf: ", "bold": true}, {"type": "text", "value": "Height 39.3 in, Width 34.9 in, Depth 13 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood in a Chestnut or Almond finish, carved scalloped door fronts, four doors with finger pulls, interior shelving, covered cable holes in the back, round bun feet fitted with levelers. Low four-door media cabinet with a deeply ribbed vertical front; top suits televisions up to 80 in; rated to 176 lbs concentrated load; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 17.5 in, Width 71 in, Depth 16 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood in a Chestnut or Almond finish, carved scalloped door fronts, four doors with finger pulls, interior shelving, covered cable holes in the back, round bun feet fitted with levelers. Low four-door media cabinet with a deeply ribbed vertical front; top suits televisions up to 80 in; rated to 176 lbs concentrated load; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 17.5 in, Width 71 in, Depth 16 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2304,7 +2304,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood with wood-grain laminate finish in Jet or Almond, three full-extension drawers, two soft-close doors, adjustable interior shelves, two round plinth bases. Long sideboard with fully rounded ends; dining buffet, living room storage, office credenza or media console; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 30.9 in, Width 70.87 in, Depth 16.93 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "5.59 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Drawer interior: ", "bold": true}, {"type": "text", "value": "Height 3.94 in, Width 13.27 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood with wood-grain laminate finish in Jet or Almond, three full-extension drawers, two soft-close doors, adjustable interior shelves, two round plinth bases. Long sideboard with fully rounded ends; dining buffet, living room storage, office credenza or media console; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 30.9 in, Width 70.87 in, Depth 16.93 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "5.59 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Drawer interior: ", "bold": true}, {"type": "text", "value": "Height 3.94 in, Width 13.27 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood in a Chestnut or Blonde finish, carved scalloped door fronts, three doors with finger pulls, interior shelving, covered cable holes in the back for media use, round bun feet fitted with levelers. Three-door sideboard with a deeply ribbed vertical front; works as buffet, media console or entry cabinet; rated to 200 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32 in, Width 54 in, Depth 19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood in a Chestnut or Blonde finish, carved scalloped door fronts, three doors with finger pulls, interior shelving, covered cable holes in the back for media use, round bun feet fitted with levelers. Three-door sideboard with a deeply ribbed vertical front; works as buffet, media console or entry cabinet; rated to 200 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32 in, Width 54 in, Depth 19.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2348,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Sturdy engineered wood in a choice of finishes. Narrow leaning, tiered ladder-frame bookcase with three open shelves over a single-door cupboard for concealed storage."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 71 in, Width 20.5 in, Depth 15 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "5.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "0.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Sturdy engineered wood in a choice of finishes. Narrow leaning, tiered ladder-frame bookcase with three open shelves over a single-door cupboard for concealed storage."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 71 in, Width 20.5 in, Depth 15 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "5.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "0.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2370,7 +2370,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood in a Cocoa or Blonde wood-grain veneer, rounded bullnose edges, two open tiers, bun feet on non-marking glides. Long low open bookcase for living room, home office or bedroom, under a window or a TV; rated to 137 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 28.5 in, Width 60 in, Depth 14 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Shelf: ", "bold": true}, {"type": "text", "value": "Height 11.5 in, Width 42.5 in, Depth 14 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood in a Cocoa or Blonde wood-grain veneer, rounded bullnose edges, two open tiers, bun feet on non-marking glides. Long low open bookcase for living room, home office or bedroom, under a window or a TV; rated to 137 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 28.5 in, Width 60 in, Depth 14 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Shelf: ", "bold": true}, {"type": "text", "value": "Height 11.5 in, Width 42.5 in, Depth 14 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2392,7 +2392,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood case with arched surround in Jet, Willow, Loden or Sand and a warm wood-grain laminate interior, four open tiers with adjustable shelves, each shelf rated to 99 lbs. Tall arch-topped open bookcase and display shelf for dining room, living room, hallway or office; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 75 in, Width 31.7 in, Depth 15.8 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Height 13.7 in, Width 30.1 in, Depth 15.2 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood case with arched surround in Jet, Willow, Loden or Sand and a warm wood-grain laminate interior, four open tiers with adjustable shelves, each shelf rated to 99 lbs. Tall arch-topped open bookcase and display shelf for dining room, living room, hallway or office; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 75 in, Width 31.7 in, Depth 15.8 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Height 13.7 in, Width 30.1 in, Depth 15.2 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Real burl wood veneer in Almond or Honey over an engineered wood core, adjustable leveling feet with non-marking pads. Square block side table with veneer wrapped across the top and sides; each figure is unique; rated to 298 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20.5 in, Width 16 in, Depth 16 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Real burl wood veneer in Almond or Honey over an engineered wood core, adjustable leveling feet with non-marking pads. Square block side table with veneer wrapped across the top and sides; each figure is unique; rated to 298 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20.5 in, Width 16 in, Depth 16 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Solid hardwood round tray top in Hazel or Cocoa with a raised rim, black iron stem, white marble cylinder base, non-marking pad. Small pedestal side table for sofa, home office, guest room or entryway; rated to 99 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20 in, Width 14 in, Depth 14 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Solid hardwood round tray top in Hazel or Cocoa with a raised rim, black iron stem, white marble cylinder base, non-marking pad. Small pedestal side table for sofa, home office, guest room or entryway; rated to 99 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20 in, Width 14 in, Depth 14 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "1 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2458,7 +2458,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Solid hardwood and engineered wood with flexible plywood drum sections, finish in Honey, Jet, Terracotta or Claret, non-marking glides. Square stacked side table of three slabs and two round drums; nightstand, end table, hall table or plant stand; rated to 77 lbs; fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20 in, Width 18 in, Depth 18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "16 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Solid hardwood and engineered wood with flexible plywood drum sections, finish in Honey, Jet, Terracotta or Claret, non-marking glides. Square stacked side table of three slabs and two round drums; nightstand, end table, hall table or plant stand; rated to 77 lbs; fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20 in, Width 18 in, Depth 18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "16 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2480,7 +2480,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Natural rattan woven over the top and pedestal in Mink or Flax, thick rolled rim. Round side table on one woven clover pedestal, top open on every side, narrow base that pulls in close to a sofa or chair arm; lightweight and easy to carry one-handed; rated to 44 lbs; comes fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20 in, Width 20 in, Depth 20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "3.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "16.1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Natural rattan woven over the top and pedestal in Mink or Flax, thick rolled rim. Round side table on one woven clover pedestal, top open on every side, narrow base that pulls in close to a sofa or chair arm; lightweight and easy to carry one-handed; rated to 44 lbs; comes fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20 in, Width 20 in, Depth 20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "3.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "16.1 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2502,7 +2502,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Natural rattan woven over the top and both pedestals in Mink or Flax, thick rolled rim. Tall, shallow oval console table on two three-lobed clover pedestals set wide apart, with open floor between for a bench or baskets; suits a hallway wall or the back of a sofa; rated to 44 lbs; light assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34 in, Width 59 in, Depth 18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "3.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "30.4 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Natural rattan woven over the top and both pedestals in Mink or Flax, thick rolled rim. Tall, shallow oval console table on two three-lobed clover pedestals set wide apart, with open floor between for a bench or baskets; suits a hallway wall or the back of a sofa; rated to 44 lbs; light assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34 in, Width 59 in, Depth 18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "3.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "30.4 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2524,7 +2524,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Real burl wood veneer in Almond or Honey over an engineered wood core, adjustable leveling feet with non-marking pads. Low round drum coffee table with veneer wrapped across the top and sides; each figure is unique; rated to 441 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 16.5 in, Width 35 in, Depth 35 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Real burl wood veneer in Almond or Honey over an engineered wood core, adjustable leveling feet with non-marking pads. Low round drum coffee table with veneer wrapped across the top and sides; each figure is unique; rated to 441 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 16.5 in, Width 35 in, Depth 35 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2722,7 +2722,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Moulded acrylic in Pewter or Citron (translucent tint), one-piece construction. Armless medallion-back dining chair with oval back and square tapering legs; 19 in seat height for a standard dining table; sturdy and durable; suits any room and outdoor use; sold singly."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35.5 in, Width 15 in, Depth 19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Moulded acrylic in Pewter or Citron (translucent tint), one-piece construction. Armless medallion-back dining chair with oval back and square tapering legs; 19 in seat height for a standard dining table; sturdy and durable; suits any room and outdoor use; sold singly."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35.5 in, Width 15 in, Depth 19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2744,7 +2744,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft, hard-wearing polyester woven fabric upholstery in Oyster or Pewter, thick dense foam padding, curved backrest, sled base of matte black stainless steel in Jet. Armless upholstered dining side chair, also suits living room, lounge or office seating; rated to 331 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32 in, Width 19 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft, hard-wearing polyester woven fabric upholstery in Oyster or Pewter, thick dense foam padding, curved backrest, sled base of matte black stainless steel in Jet. Armless upholstered dining side chair, also suits living room, lounge or office seating; rated to 331 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32 in, Width 19 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2766,7 +2766,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Moulded acrylic in Jet (opaque gloss) or Crystal (clear), one-piece construction. Armless medallion-back dining chair with oval back and square tapering legs; 18.5 in seat height for a standard dining table; sturdy and durable; suits any room and outdoor use; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35.5 in, Width 15 in, Depth 19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Moulded acrylic in Jet (opaque gloss) or Crystal (clear), one-piece construction. Armless medallion-back dining chair with oval back and square tapering legs; 18.5 in seat height for a standard dining table; sturdy and durable; suits any room and outdoor use; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35.5 in, Width 15 in, Depth 19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2788,7 +2788,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Solid hardwood frame in Honey, woven faux rattan back panel, foam-padded seat in heathered woven fabric in Heathered Ink, Heathered Dove or Heathered Cream, tapered legs, foot glides. Armless woven-back dining chairs; each rated to 507 lbs; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.4 in, Width 19.5 in, Depth 23 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Solid hardwood frame in Honey, woven faux rattan back panel, foam-padded seat in heathered woven fabric in Heathered Ink, Heathered Dove or Heathered Cream, tapered legs, foot glides. Armless woven-back dining chairs; each rated to 507 lbs; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.4 in, Width 19.5 in, Depth 23 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2810,7 +2810,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven fabric upholstery in Oyster or Malachite, dense foam padding, solid wood frame, dark-finished wooden legs, non-marking foot glides, silver-toned nailhead trim. Tall flared-back Parsons-style dining chair; set of two chairs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 40 in, Width 19.5 in, Depth 23.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "23.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "6 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven fabric upholstery in Oyster or Malachite, dense foam padding, solid wood frame, dark-finished wooden legs, non-marking foot glides, silver-toned nailhead trim. Tall flared-back Parsons-style dining chair; set of two chairs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 40 in, Width 19.5 in, Depth 23.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "23.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "6 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2832,7 +2832,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Kiln-dried wood frame, padded seat and tall back, removable tailored slipcover in linen-blend fabric in Olive, Sand, Bark, Aegean or Cream, or in striped fabric in Mushroom Stripe, Charcoal Stripe or Chambray Stripe, concealed casters for rolling the chair into place. Straight-backed slipcovered dining side chair for dining room, kitchen table or entryway; single chair; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.5 in, Width 18.5 in, Depth 25 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "4 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Kiln-dried wood frame, padded seat and tall back, removable tailored slipcover in linen-blend fabric in Olive, Sand, Bark, Aegean or Cream, or in striped fabric in Mushroom Stripe, Charcoal Stripe or Chambray Stripe, concealed casters for rolling the chair into place. Straight-backed slipcovered dining side chair for dining room, kitchen table or entryway; single chair; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.5 in, Width 18.5 in, Depth 25 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "4 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2854,7 +2854,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood blend with a wood-grain veneer finish in Chestnut or a matte painted finish, rounded waterfall edges, fluted doors and sides, four push-to-open doors, adjustable interior shelves, covered cord holes, adjustable levelers. Long fluted sideboard for buffet, media or hall storage; arrives fully assembled; weight capacity not stated."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 31 in, Width 70 in, Depth 18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood blend with a wood-grain veneer finish in Chestnut or a matte painted finish, rounded waterfall edges, fluted doors and sides, four push-to-open doors, adjustable interior shelves, covered cord holes, adjustable levelers. Long fluted sideboard for buffet, media or hall storage; arrives fully assembled; weight capacity not stated."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 31 in, Width 70 in, Depth 18.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2876,7 +2876,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood frame with natural rattan, four shelves, open back, raised legs, non-marking foot caps. Tall arched open-back bookcase for living room or office; slight natural variation in rattan colour and pattern; arrives fully assembled; weight capacity not stated."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 67.9 in, Width 29.8 in, Depth 13.7 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Height 14.3 in, Width 27.3 in, Depth 13.7 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Shelf: ", "bold": true}, {"type": "text", "value": "Height 1.2 in, Width 27.2 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood frame with natural rattan, four shelves, open back, raised legs, non-marking foot caps. Tall arched open-back bookcase for living room or office; slight natural variation in rattan colour and pattern; arrives fully assembled; weight capacity not stated."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 67.9 in, Width 29.8 in, Depth 13.7 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Height 14.3 in, Width 27.3 in, Depth 13.7 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Shelf: ", "bold": true}, {"type": "text", "value": "Height 1.2 in, Width 27.2 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2898,7 +2898,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft woven polyester upholstery in Dove, Teal, Oyster or Pewter, dense foam (5 in cushion) over sinuous spring seat support, deep button tufting on the inside back, solid hardwood legs braced by stretchers that serve as a footrest, non-marking caps. Counter-height stool with a tall winged back; 26.5 in seat height; rated to 500 lbs each; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 42 in, Width 21 in, Depth 19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "26.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft woven polyester upholstery in Dove, Teal, Oyster or Pewter, dense foam (5 in cushion) over sinuous spring seat support, deep button tufting on the inside back, solid hardwood legs braced by stretchers that serve as a footrest, non-marking caps. Counter-height stool with a tall winged back; 26.5 in seat height; rated to 500 lbs each; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 42 in, Width 21 in, Depth 19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "26.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2920,7 +2920,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Solid hardwood frame in Blonde finish, Jet or Flax rope seat woven in a basket pattern, leg rungs that serve as footrests, side supports, non-marking foot pads. Backless bar stool with a gently dished seat; 29.5 in seat height for a bar-height counter or home bar; each stool rated to 331 lbs; for kitchens, breakfast nooks, bar areas, dining counters and entertainment rooms; assembly required; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 29.5 in, Width 20 in, Depth 18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "29.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Solid hardwood frame in Blonde finish, Jet or Flax rope seat woven in a basket pattern, leg rungs that serve as footrests, side supports, non-marking foot pads. Backless bar stool with a gently dished seat; 29.5 in seat height for a bar-height counter or home bar; each stool rated to 331 lbs; for kitchens, breakfast nooks, bar areas, dining counters and entertainment rooms; assembly required; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 29.5 in, Width 20 in, Depth 18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "29.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2942,7 +2942,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft woven fabric upholstery in Mink, Charcoal or Oyster, padded seat, bentwood frame, metal foot rail, foot pins that protect floors. Bar-height barrel-back stool with a curved open back and arms that run to the floor as solid sides; 28.5 in seat height for a standard home bar; rated to 300 lbs; arrives fully assembled; sold singly."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 41 in, Width 22 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "28.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "35 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Back height above seat: ", "bold": true}, {"type": "text", "value": "12 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft woven fabric upholstery in Mink, Charcoal or Oyster, padded seat, bentwood frame, metal foot rail, foot pins that protect floors. Bar-height barrel-back stool with a curved open back and arms that run to the floor as solid sides; 28.5 in seat height for a standard home bar; rated to 300 lbs; arrives fully assembled; sold singly."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 41 in, Width 22 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "28.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "35 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Back height above seat: ", "bold": true}, {"type": "text", "value": "12 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2964,7 +2964,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven fabric upholstery in Oyster, Bark, Smoke or Dove, dense foam padding in seat and back, deep button-tufted curved back, wooden legs in a dark finish, non-marking foot caps. Tall curved-back upholstered dining chair; set of four chairs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 37.5 in, Width 24.5 in, Depth 18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "21.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven fabric upholstery in Oyster, Bark, Smoke or Dove, dense foam padding in seat and back, deep button-tufted curved back, wooden legs in a dark finish, non-marking foot caps. Tall curved-back upholstered dining chair; set of four chairs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 37.5 in, Width 24.5 in, Depth 18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "21.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -2986,7 +2986,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood bentwood frame in Jet or Hazel with a durable polyurethane finish, round wooden seat, leg brace ring, non-marking plastic glides. Bentwood dining side chair for dining rooms, kitchens and café-style seating; no assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35 in, Width 15 in, Depth 20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "15.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood bentwood frame in Jet or Hazel with a durable polyurethane finish, round wooden seat, leg brace ring, non-marking plastic glides. Bentwood dining side chair for dining rooms, kitchens and café-style seating; no assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35 in, Width 15 in, Depth 20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "15.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3008,7 +3008,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft durable polyester fabric upholstery in Oyster, Charcoal or Dove, dense foam padding, solid hardwood legs and curved side rails in Jet, plastic foot pins. Upholstered dining side chairs with curved rails linking seat and back, also suited as accent chairs in living rooms, offices, bedrooms or entries; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 38 in, Width 21.5 in, Depth 24.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "20.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft durable polyester fabric upholstery in Oyster, Charcoal or Dove, dense foam padding, solid hardwood legs and curved side rails in Jet, plastic foot pins. Upholstered dining side chairs with curved rails linking seat and back, also suited as accent chairs in living rooms, offices, bedrooms or entries; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 38 in, Width 21.5 in, Depth 24.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "20.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in Navy or Pewter, deep button tufting, French piping, dense foam padding, sinuous spring seat support, carved cabriole legs in a weathered Driftwood finish, plastic foot caps. Wingback armchair for dining or for accent use in living room, bedroom, home office or entryway; 20 in seat height; rated to 300 lbs; single chair."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 39.5 in, Width 28.5 in, Depth 25.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "20.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in Navy or Pewter, deep button tufting, French piping, dense foam padding, sinuous spring seat support, carved cabriole legs in a weathered Driftwood finish, plastic foot caps. Wingback armchair for dining or for accent use in living room, bedroom, home office or entryway; 20 in seat height; rated to 300 lbs; single chair."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 39.5 in, Width 28.5 in, Depth 25.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "20.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3052,7 +3052,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame, soft woven fabric upholstery in Oyster or Pewter, dense foam padding, deep button tufting on the inside back, non-marking floor glides. Tall winged dining chairs with curved backs; 19 in seat height; set of four."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 38.5 in, Width 21 in, Depth 26.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame, soft woven fabric upholstery in Oyster or Pewter, dense foam padding, deep button tufting on the inside back, non-marking floor glides. Tall winged dining chairs with curved backs; 19 in seat height; set of four."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 38.5 in, Width 21 in, Depth 26.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3074,7 +3074,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Solid hardwood frame in Jet or Almond, woven cane backrest, bentwood seat with wood-grain veneer, non-marking foot caps. Armless cane-back dining chair, also suited to living room, office or entryway; each rated to 330 lbs; set of 2."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 31 in, Width 16.5 in, Depth 23.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Solid hardwood frame in Jet or Almond, woven cane backrest, bentwood seat with wood-grain veneer, non-marking foot caps. Armless cane-back dining chair, also suited to living room, office or entryway; each rated to 330 lbs; set of 2."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 31 in, Width 16.5 in, Depth 23.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3096,7 +3096,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft woven fabric upholstery in a choice of five colours, dense foam padding (4 in seat cushion), deep button tufting on the inside back, solid hardwood and engineered wood frame, non-marking floor glides. Tall winged dining chair on Parsons lines with a gently curved back; 19.5 in seat height; suits a dining room, home office, entryway or living room."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 38.5 in, Width 25 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft woven fabric upholstery in a choice of five colours, dense foam padding (4 in seat cushion), deep button tufting on the inside back, solid hardwood and engineered wood frame, non-marking floor glides. Tall winged dining chair on Parsons lines with a gently curved back; 19.5 in seat height; suits a dining room, home office, entryway or living room."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 38.5 in, Width 25 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3118,7 +3118,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven polyester fabric upholstery in a choice of three soft neutrals, foam-padded seat, nailhead trim, tapered wooden legs in a dark finish, non-marking foot caps. Upholstered dining chair with waisted back and low flared sides, for classic or modern dining rooms, plus a home office desk, a hall or a living room."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 36 in, Width 22 in, Depth 25 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven polyester fabric upholstery in a choice of three soft neutrals, foam-padded seat, nailhead trim, tapered wooden legs in a dark finish, non-marking foot caps. Upholstered dining chair with waisted back and low flared sides, for classic or modern dining rooms, plus a home office desk, a hall or a living room."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 36 in, Width 22 in, Depth 25 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3140,7 +3140,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid wood frame in Jet or Honey, woven faux cane back panel, dense foam seat upholstered in smooth vegan leather in Caramel or Jet, non-marking foot glides. Tall-backed dining side chair with a squared frame and square legs, also at home as an accent chair; rated to 551 lbs; set of two; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 39 in, Width 19.7 in, Depth 23.2 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.425 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.915 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid wood frame in Jet or Honey, woven faux cane back panel, dense foam seat upholstered in smooth vegan leather in Caramel or Jet, non-marking foot glides. Tall-backed dining side chair with a squared frame and square legs, also at home as an accent chair; rated to 551 lbs; set of two; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 39 in, Width 19.7 in, Depth 23.2 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.425 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.915 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3162,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood frame in Honey, Oyster or Jet, woven rattan cane back panel, dense foam seat upholstered in fabric in Heathered Cream or Pewter, non-marking floor glides. Cane-back dining armchair with short open arms and slim legs; also suits a living room or home office; rated to 330 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.5 in, Width 20.6 in, Depth 20.9 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "2 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood frame in Honey, Oyster or Jet, woven rattan cane back panel, dense foam seat upholstered in fabric in Heathered Cream or Pewter, non-marking floor glides. Cane-back dining armchair with short open arms and slim legs; also suits a living room or home office; rated to 330 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.5 in, Width 20.6 in, Depth 20.9 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "2 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3184,7 +3184,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft slubbed fabric upholstery in Flax, Mink or Cream, foam padding, solid wood frame, solid wood legs in a natural or dark finish, non-marking glides. Tailored upholstered dining armchair with sloping arms, also an accent chair for living rooms; rated to 300 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.5 in, Width 23.5 in, Depth 24.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "25 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height above seat: ", "bold": true}, {"type": "text", "value": "4.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft slubbed fabric upholstery in Flax, Mink or Cream, foam padding, solid wood frame, solid wood legs in a natural or dark finish, non-marking glides. Tailored upholstered dining armchair with sloping arms, also an accent chair for living rooms; rated to 300 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.5 in, Width 23.5 in, Depth 24.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "25 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height above seat: ", "bold": true}, {"type": "text", "value": "4.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3206,7 +3206,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame, foam-padded vegan leather seat in Stone or Jet, curved top rail with angled arms, splayed legs, non-marking floor pins. Mid-century style dining armchair for dining room or kitchen, also an accent chair; rated to 300 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 27.5 in, Width 22.5 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "27 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height above seat: ", "bold": true}, {"type": "text", "value": "8.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame, foam-padded vegan leather seat in Stone or Jet, curved top rail with angled arms, splayed legs, non-marking floor pins. Mid-century style dining armchair for dining room or kitchen, also an accent chair; rated to 300 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 27.5 in, Width 22.5 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "27 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height above seat: ", "bold": true}, {"type": "text", "value": "8.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3228,7 +3228,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft bouclé upholstery in Cream or Dove spun from recycled plastic bottles, fabric certified to a recognised textile safety standard, fully padded body, arched high back, waterfall-front base, non-marking floor glides. Armless slipper-style dining chair, also a desk or bedroom chair; rated to 300 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.5 in, Width 21.5 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "2 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft bouclé upholstery in Cream or Dove spun from recycled plastic bottles, fabric certified to a recognised textile safety standard, fully padded body, arched high back, waterfall-front base, non-marking floor glides. Armless slipper-style dining chair, also a desk or bedroom chair; rated to 300 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.5 in, Width 21.5 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "2 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3250,7 +3250,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in Pewter or Chambray, dense foam padding, wood and plywood frame, splayed brushed Brass-tone stainless steel legs with non-marking caps, Brass-tone pull on the outer back for drawing the chair out. Scoop-back upholstered dining armchair with low sloping arms; outer back finished in vertical pleats; also suits a desk, vanity, bedroom, living room or entryway."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34 in, Width 25 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in Pewter or Chambray, dense foam padding, wood and plywood frame, splayed brushed Brass-tone stainless steel legs with non-marking caps, Brass-tone pull on the outer back for drawing the chair out. Scoop-back upholstered dining armchair with low sloping arms; outer back finished in vertical pleats; also suits a desk, vanity, bedroom, living room or entryway."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34 in, Width 25 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3272,7 +3272,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood frame in Jet or Blonde, woven synthetic rattan cane seat inset, curved top rail with spindle back, tapered splayed legs with stretchers. Spindle-back dining chairs for kitchen, dining room or breakfast nook, set of two; rated to 400 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 30 in, Width 21 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "17.9 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.9 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood frame in Jet or Blonde, woven synthetic rattan cane seat inset, curved top rail with spindle back, tapered splayed legs with stretchers. Spindle-back dining chairs for kitchen, dining room or breakfast nook, set of two; rated to 400 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 30 in, Width 21 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "17.9 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.9 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3294,7 +3294,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Solid kiln-dried hardwood frame in Hazel, soft durable woven fabric upholstery in Cream, Charcoal or Stone, padded seat and low back, non-marking glides. Compact armless upholstered dining chair for kitchens, dining rooms and small spaces, also a side or accent chair; rated to 300 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32 in, Width 19.5 in, Depth 21.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Back height above seat: ", "bold": true}, {"type": "text", "value": "13 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "3 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Solid kiln-dried hardwood frame in Hazel, soft durable woven fabric upholstery in Cream, Charcoal or Stone, padded seat and low back, non-marking glides. Compact armless upholstered dining chair for kitchens, dining rooms and small spaces, also a side or accent chair; rated to 300 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32 in, Width 19.5 in, Depth 21.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Back height above seat: ", "bold": true}, {"type": "text", "value": "13 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "3 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3316,7 +3316,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Textured slub-weave fabric upholstery in Oyster, Jet, Mink, Stone or Ink, dense foam padding, sturdy internal frame, non-marking floor glides. Armless slipper dining chair with a tall back and a waterfall seat front that folds down to the floor; 19.3 in seat height for a standard dining table; rated to 300 lbs; for kitchen tables, vanities and living rooms; arrives fully assembled; single chair."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35.4 in, Width 19.7 in, Depth 24.2 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.3 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.7 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "3.2 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Textured slub-weave fabric upholstery in Oyster, Jet, Mink, Stone or Ink, dense foam padding, sturdy internal frame, non-marking floor glides. Armless slipper dining chair with a tall back and a waterfall seat front that folds down to the floor; 19.3 in seat height for a standard dining table; rated to 300 lbs; for kitchen tables, vanities and living rooms; arrives fully assembled; single chair."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35.4 in, Width 19.7 in, Depth 24.2 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.3 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.7 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "3.2 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3338,7 +3338,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in Cream, Fawn, Aegean, Truffle or Claret, dense foam padding, sturdy internal frame, non-marking floor glides. Armless slipper dining chair with a tall back and a waterfall seat front that folds down to the floor; 19.5 in seat height for a standard dining table; each chair rated to 300 lbs; suits dining rooms, vanities and living rooms; arrives fully assembled; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35.5 in, Width 19.5 in, Depth 24.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "3 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in Cream, Fawn, Aegean, Truffle or Claret, dense foam padding, sturdy internal frame, non-marking floor glides. Armless slipper dining chair with a tall back and a waterfall seat front that folds down to the floor; 19.5 in seat height for a standard dining table; each chair rated to 300 lbs; suits dining rooms, vanities and living rooms; arrives fully assembled; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35.5 in, Width 19.5 in, Depth 24.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "3 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3360,7 +3360,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood frame in Blonde, Chestnut or Charcoal, woven rope seat and back in Flax or Jet, curved back rail, leg stretchers. Armless dining chair with an open woven back, for dining rooms, kitchens, offices or occasional seating; rated to 330 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32 in, Width 20 in, Depth 20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "14.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood frame in Blonde, Chestnut or Charcoal, woven rope seat and back in Flax or Jet, curved back rail, leg stretchers. Armless dining chair with an open woven back, for dining rooms, kitchens, offices or occasional seating; rated to 330 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32 in, Width 20 in, Depth 20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "14.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3382,7 +3382,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Performance fabric upholstery in Mink, Oyster, Moss or Flax that repels water-based spills, or striped fabric in Oat Ticking Stripe (blot with a clean cloth; diluted dish soap for stubborn marks), floor-length skirted cover with pleated corners, resilient foam seat, back and seat cushions that lift off, hardwood frame, adjustable levelling feet. Slipcovered dining armchair for dining rooms and breakfast nooks; rated to 300 lb; sold singly; light assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.5 in, Width 25 in, Depth 26 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "15.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "24.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height above seat: ", "bold": true}, {"type": "text", "value": "5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Performance fabric upholstery in Mink, Oyster, Moss or Flax that repels water-based spills, or striped fabric in Oat Ticking Stripe (blot with a clean cloth; diluted dish soap for stubborn marks), floor-length skirted cover with pleated corners, resilient foam seat, back and seat cushions that lift off, hardwood frame, adjustable levelling feet. Slipcovered dining armchair for dining rooms and breakfast nooks; rated to 300 lb; sold singly; light assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.5 in, Width 25 in, Depth 26 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "15.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "24.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height above seat: ", "bold": true}, {"type": "text", "value": "5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3404,7 +3404,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood-grain laminate case in Jet, Cream, Almond or Cocoa with edge trim, tapered wood legs, soft-close hinges, brass-toned metal ring pulls, non-marking foot pads. Tall arch-topped bookcase with open upper shelving (two fixed and two adjustable shelves) and a two-door lower cupboard whose two adjustable shelves form four compartments; each shelf holds up to 44 lb; for a living room, dining room or hallway; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 74.1 in, Width 39.37 in, Depth 16.54 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood-grain laminate case in Jet, Cream, Almond or Cocoa with edge trim, tapered wood legs, soft-close hinges, brass-toned metal ring pulls, non-marking foot pads. Tall arch-topped bookcase with open upper shelving (two fixed and two adjustable shelves) and a two-door lower cupboard whose two adjustable shelves form four compartments; each shelf holds up to 44 lb; for a living room, dining room or hallway; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 74.1 in, Width 39.37 in, Depth 16.54 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3426,7 +3426,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood frame with a laminate wood-grain surface in Hazel or Almond, two slatted doors with press-to-open latches and soft-close hinges, one adjustable interior shelf, recessed plinth base. Compact two-door accent cabinet for entryway, hallway, dining room or living room; works as a small buffet, bar or media console; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 29.7 in, Width 35.3 in, Depth 16.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Height 25.8 in, Width 34 in, Depth 16 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood frame with a laminate wood-grain surface in Hazel or Almond, two slatted doors with press-to-open latches and soft-close hinges, one adjustable interior shelf, recessed plinth base. Compact two-door accent cabinet for entryway, hallway, dining room or living room; works as a small buffet, bar or media console; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 29.7 in, Width 35.3 in, Depth 16.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Height 25.8 in, Width 34 in, Depth 16 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3448,7 +3448,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood with matte wood-grain finish in Almond or Jet, two drawers, two soft-close cupboard doors, adjustable shelf, three covered rear cable-management openings, two round plinth bases. Long, low media cabinet with rounded ends for use under a wall-mounted TV; rated to 200 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 22.5 in, Width 70.9 in, Depth 17 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Height 13.8 in, Width 22.9 in, Depth 15.4 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood with matte wood-grain finish in Almond or Jet, two drawers, two soft-close cupboard doors, adjustable shelf, three covered rear cable-management openings, two round plinth bases. Long, low media cabinet with rounded ends for use under a wall-mounted TV; rated to 200 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 22.5 in, Width 70.9 in, Depth 17 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Height 13.8 in, Width 22.9 in, Depth 15.4 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3470,7 +3470,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood construction with Chestnut or Jet wood grain finish, vertical fluting on front and sides, rounded ends, four handle-free press-to-open doors, interior storage bays with a movable centre shelf, rear cable opening for media use, floor-protecting foot caps. Long curved-end sideboard for use as a buffet, a console under a wall-mounted TV or a credenza; top rated to 254 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 24.73 in, Width 75.35 in, Depth 16.97 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood construction with Chestnut or Jet wood grain finish, vertical fluting on front and sides, rounded ends, four handle-free press-to-open doors, interior storage bays with a movable centre shelf, rear cable opening for media use, floor-protecting foot caps. Long curved-end sideboard for use as a buffet, a console under a wall-mounted TV or a credenza; top rated to 254 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 24.73 in, Width 75.35 in, Depth 16.97 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3492,7 +3492,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood in Chestnut or Blonde finish, carved scalloped door fronts, four doors with finger pulls, interior shelving, covered cable holes in the back for media use, round bun feet fitted with levelers. Four-door sideboard with a deeply ribbed vertical front; works as buffet, media console or entry cabinet; rated to 200 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32 in, Width 72 in, Depth 19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood in Chestnut or Blonde finish, carved scalloped door fronts, four doors with finger pulls, interior shelving, covered cable holes in the back for media use, round bun feet fitted with levelers. Four-door sideboard with a deeply ribbed vertical front; works as buffet, media console or entry cabinet; rated to 200 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32 in, Width 72 in, Depth 19.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3514,7 +3514,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Sturdy engineered wood in a choice of finishes. Wide leaning, tiered ladder-frame bookcase with three open shelves over a two-door cupboard for concealed storage."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 71 in, Width 32.5 in, Depth 15.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "5.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "0.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Sturdy engineered wood in a choice of finishes. Wide leaning, tiered ladder-frame bookcase with three open shelves over a two-door cupboard for concealed storage."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 71 in, Width 32.5 in, Depth 15.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "5.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "0.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3536,7 +3536,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood frame and four open wood shelves in Blonde, Jet or Chestnut, matching arched frames front and back, open back and sides, non-marking glides. Tall, narrow open bookcase about 6 ft high and 2 ft wide, for books, collected pieces and display; shelves hold up to 220 lbs in all; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 72.1 in, Width 24 in, Depth 14.1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Shelf: ", "bold": true}, {"type": "text", "value": "Height 1.2 in, Width 24 in, Depth 14.1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood frame and four open wood shelves in Blonde, Jet or Chestnut, matching arched frames front and back, open back and sides, non-marking glides. Tall, narrow open bookcase about 6 ft high and 2 ft wide, for books, collected pieces and display; shelves hold up to 220 lbs in all; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 72.1 in, Width 24 in, Depth 14.1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Shelf: ", "bold": true}, {"type": "text", "value": "Height 1.2 in, Width 24 in, Depth 14.1 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3558,7 +3558,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Bent natural rattan frame, three woven rattan shelves spaced about 20 in apart, fan-spindle arched top, plastic floor glides. Tall narrow arched bookcase for bedroom, living room or sunroom; rated to 44 lbs per shelf, 132 lbs total; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 68 in, Width 30 in, Depth 14 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "11.1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Bent natural rattan frame, three woven rattan shelves spaced about 20 in apart, fan-spindle arched top, plastic floor glides. Tall narrow arched bookcase for bedroom, living room or sunroom; rated to 44 lbs per shelf, 132 lbs total; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 68 in, Width 30 in, Depth 14 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "11.1 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3580,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Solid hardwood and wood veneer in Blonde, Jet or Chestnut finish, round top with thick edge, cross base of two interlocking full-height panels, adjustable levelling feet that protect the floor. Small round side table for sofa ends, bedsides, entries and halls; rated to 132 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 18 in, Width 15.5 in, Depth 15.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "17 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Solid hardwood and wood veneer in Blonde, Jet or Chestnut finish, round top with thick edge, cross base of two interlocking full-height panels, adjustable levelling feet that protect the floor. Small round side table for sofa ends, bedsides, entries and halls; rated to 132 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 18 in, Width 15.5 in, Depth 15.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "17 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "1 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3602,7 +3602,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Iron construction, raised-rim round tray top, conical pedestal base, non-marking pad, Pewter, Jet or Brass finish. Small round side table for beside a sofa or lounge chair, home office, entryway or hallway; rated to 88 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 21 in, Width 16 in, Depth 16 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Iron construction, raised-rim round tray top, conical pedestal base, non-marking pad, Pewter, Jet or Brass finish. Small round side table for beside a sofa or lounge chair, home office, entryway or hallway; rated to 88 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 21 in, Width 16 in, Depth 16 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "1 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3624,7 +3624,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood carved in four stacked rounded tiers, finish in Jet (wire-brushed) or Honey, non-marking foam pad. Small round sculptural side table for drinks, plants or small spaces; rated to 50 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20 in, Width 17 in, Depth 17 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood carved in four stacked rounded tiers, finish in Jet (wire-brushed) or Honey, non-marking foam pad. Small round sculptural side table for drinks, plants or small spaces; rated to 50 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20 in, Width 17 in, Depth 17 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3646,7 +3646,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood in Chestnut or Almond, adjustable non-marking feet for levelling on uneven floors. Slim rectangular console or sofa table with a board top and two tall split-panel legs, rounded edges; for entryway, hallway, living room or dining room; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 30 in, Width 46 in, Depth 14 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood in Chestnut or Almond, adjustable non-marking feet for levelling on uneven floors. Slim rectangular console or sofa table with a board top and two tall split-panel legs, rounded edges; for entryway, hallway, living room or dining room; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 30 in, Width 46 in, Depth 14 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "1 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3668,7 +3668,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Finish in Chestnut wood grain, Oyster or Jet, stepped-profile frame with integrated side panels and nested grooves around the inner opening. Long, shallow console table for an entry, hallway or behind a sofa; tall top near kitchen-counter level; open floor beneath for a bench; top rated to 110 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.1 in, Width 63 in, Depth 16 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "28.6 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Finish in Chestnut wood grain, Oyster or Jet, stepped-profile frame with integrated side panels and nested grooves around the inner opening. Long, shallow console table for an entry, hallway or behind a sofa; tall top near kitchen-counter level; open floor beneath for a bench; top rated to 110 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.1 in, Width 63 in, Depth 16 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "28.6 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3690,7 +3690,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood in Jet or Chestnut. Round coffee table with a raised-lip tray top on a solid drum pedestal base; sized for small living rooms and apartments; rated to 156 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 17.5 in, Width 30 in, Depth 30 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood in Jet or Chestnut. Round coffee table with a raised-lip tray top on a solid drum pedestal base; sized for small living rooms and apartments; rated to 156 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 17.5 in, Width 30 in, Depth 30 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3844,7 +3844,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Moulded acrylic in Jet (opaque gloss) or Crystal (clear), one-piece construction. Armless medallion-back dining chair with oval back and square tapering legs; 19 in seat height for a standard dining table; sturdy and durable; suits any room and outdoor use; sold singly."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35.5 in, Width 15 in, Depth 19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Moulded acrylic in Jet (opaque gloss) or Crystal (clear), one-piece construction. Armless medallion-back dining chair with oval back and square tapering legs; 19 in seat height for a standard dining table; sturdy and durable; suits any room and outdoor use; sold singly."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35.5 in, Width 15 in, Depth 19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3866,7 +3866,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Moulded acrylic in Cobalt, Blush or Pewter tint (translucent), one-piece construction. Medallion-back dining armchair with oval back, curved arms and square tapering legs; 18.5 in seat height for a standard dining table; sturdy and durable; suits any room and outdoor use; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 36 in, Width 21 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "26 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Moulded acrylic in Cobalt, Blush or Pewter tint (translucent), one-piece construction. Medallion-back dining armchair with oval back, curved arms and square tapering legs; 18.5 in seat height for a standard dining table; sturdy and durable; suits any room and outdoor use; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 36 in, Width 21 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "26 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3888,7 +3888,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood frame and wooden seat in a choice of finishes, non-marking foot caps. Café-style dining chair with a curved top rail, crossed back splats and splayed legs braced by curved hoops beneath the seat; 18.5 in seat height; rated to 330 lbs; for dining room or kitchen, also a desk or living room side chair."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.5 in, Width 19.5 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood frame and wooden seat in a choice of finishes, non-marking foot caps. Café-style dining chair with a curved top rail, crossed back splats and splayed legs braced by curved hoops beneath the seat; 18.5 in seat height; rated to 330 lbs; for dining room or kitchen, also a desk or living room side chair."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.5 in, Width 19.5 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3910,7 +3910,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Powder-coated metal frame in Jet, textured woven fabric upholstery in Cream, Dove or Cobalt certified to a textile safety standard, padded seat and curved barrel back, adjustable non-marking glides. Open-back dining armchair with angular metal frame, also suited to desk or accent use; rated to 300 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 31.5 in, Width 21.5 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "26 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Powder-coated metal frame in Jet, textured woven fabric upholstery in Cream, Dove or Cobalt certified to a textile safety standard, padded seat and curved barrel back, adjustable non-marking glides. Open-back dining armchair with angular metal frame, also suited to desk or accent use; rated to 300 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 31.5 in, Width 21.5 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "26 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3932,7 +3932,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven polyester fabric upholstery in Oyster or Dove, foam-padded seat, nailhead trim, tapered wooden legs in a dark finish, non-marking foot caps. Upholstered dining chair with waisted back and low flared sides, for classic or modern dining rooms; set of two chairs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 36 in, Width 25 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven polyester fabric upholstery in Oyster or Dove, foam-padded seat, nailhead trim, tapered wooden legs in a dark finish, non-marking foot caps. Upholstered dining chair with waisted back and low flared sides, for classic or modern dining rooms; set of two chairs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 36 in, Width 25 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "22 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3954,7 +3954,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Honey or Jet, natural woven paper cord seat, curved back panel, open arms, X-shaped seat stretcher, non-marking floor glides. Dining armchair for kitchen or dining room; seat height 18.1 in; each rated to 497 lbs; set of two armchairs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33 in, Width 22 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18.7 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Honey or Jet, natural woven paper cord seat, curved back panel, open arms, X-shaped seat stretcher, non-marking floor glides. Dining armchair for kitchen or dining room; seat height 18.1 in; each rated to 497 lbs; set of two armchairs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33 in, Width 22 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18.7 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3976,7 +3976,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Sturdy engineered wood finished in Almond, Hazel or White. Two-piece home office set: a leaning, tiered ladder-frame desk with a work surface, three shelves above it and a pair of pull-out drawers, plus a narrow bookcase with three open shelves over a single-door cupboard for concealed storage."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Desk: Height 71 in, Width 49 in, Depth 18.5 in; Bookcase: Height 71 in, Width 20.5 in, Depth 15 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "5.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "0.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Sturdy engineered wood finished in Almond, Hazel or White. Two-piece home office set: a leaning, tiered ladder-frame desk with a work surface, three shelves above it and a pair of pull-out drawers, plus a narrow bookcase with three open shelves over a single-door cupboard for concealed storage."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Desk: Height 71 in, Width 49 in, Depth 18.5 in; Bookcase: Height 71 in, Width 20.5 in, Depth 15 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "5.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "0.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Faux marble top in Jet or White, bevelled edge, tapered metal pedestal stem and disc foot in White, Jet or Brass with a finish that resists chips, non-marking felt floor pad. Round single-stem pedestal side table about 20 in high, level with most sofa arms; for living room, lounge corner, bedside, home office or entryway; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20.5 in, Width 19.5 in, Depth 19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Faux marble top in Jet or White, bevelled edge, tapered metal pedestal stem and disc foot in White, Jet or Brass with a finish that resists chips, non-marking felt floor pad. Round single-stem pedestal side table about 20 in high, level with most sofa arms; for living room, lounge corner, bedside, home office or entryway; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20.5 in, Width 19.5 in, Depth 19.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Textured woven fabric upholstery in Stone, Cream, Fern or Navy, certified free of harmful substances, padded seat and rounded back, polished Chrome-finish metal frame forming supportive arms and a sled base, adjustable non-marking glides. Barrel-back counter stool with a 26 in seat height for kitchen islands and counter-height tables; rated to 300 lbs; single stool; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 37 in, Width 19.5 in, Depth 19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "26 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "33.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Textured woven fabric upholstery in Stone, Cream, Fern or Navy, certified free of harmful substances, padded seat and rounded back, polished Chrome-finish metal frame forming supportive arms and a sled base, adjustable non-marking glides. Barrel-back counter stool with a 26 in seat height for kitchen islands and counter-height tables; rated to 300 lbs; single stool; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 37 in, Width 19.5 in, Depth 19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "26 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "33.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4042,7 +4042,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in Moss, Claret, Fawn, Cream or Truffle, padded seat, bentwood frame, metal foot rail, foot pins that protect floors. Counter-height barrel-back stool with a curved open back and arms that run to the floor as solid sides; 25 in seat height for a kitchen island or counter-height table; rated to 300 lbs; arrives fully assembled; sold singly."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 37 in, Width 22 in, Depth 21.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "25 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "31 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Back height above seat: ", "bold": true}, {"type": "text", "value": "12 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in Moss, Claret, Fawn, Cream or Truffle, padded seat, bentwood frame, metal foot rail, foot pins that protect floors. Counter-height barrel-back stool with a curved open back and arms that run to the floor as solid sides; 25 in seat height for a kitchen island or counter-height table; rated to 300 lbs; arrives fully assembled; sold singly."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 37 in, Width 22 in, Depth 21.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "25 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "31 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Back height above seat: ", "bold": true}, {"type": "text", "value": "12 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4064,7 +4064,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Honey or Jet, natural woven paper cord seat, supportive back panel, X-shaped seat stretcher, non-marking floor glides. Bar-height stool for bar counters and pub tables; seat height 28.7 in; each rated to 517 lbs; set of two stools; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 42 in, Width 19 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "28.7 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Width 15 in, Depth 15 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Honey or Jet, natural woven paper cord seat, supportive back panel, X-shaped seat stretcher, non-marking floor glides. Bar-height stool for bar counters and pub tables; seat height 28.7 in; each rated to 517 lbs; set of two stools; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 42 in, Width 19 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "28.7 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Width 15 in, Depth 15 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4086,7 +4086,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frames in Chestnut finish, broad curved top rail, tapered legs with stretchers, foam-cushioned seats covered in faux leather that wipes clean, in a choice of two shades. Set of two mid-century style dining side chairs; seat height 18 in."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 29 in, Width 21.5 in, Depth 19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "15.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frames in Chestnut finish, broad curved top rail, tapered legs with stretchers, foam-cushioned seats covered in faux leather that wipes clean, in a choice of two shades. Set of two mid-century style dining side chairs; seat height 18 in."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 29 in, Width 21.5 in, Depth 19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "15.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4108,7 +4108,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frames, tapered legs and bracing stretchers in Jet or Honey finish, woven paper cord seats that are soft, static-free and hard-wearing. Two spindle-back dining side chairs, each with a deep curved top rail, for dining room, kitchen or living area; seat height 18.5 in; each rated to 286 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 31.5 in, Width 45 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "15.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frames, tapered legs and bracing stretchers in Jet or Honey finish, woven paper cord seats that are soft, static-free and hard-wearing. Two spindle-back dining side chairs, each with a deep curved top rail, for dining room, kitchen or living area; seat height 18.5 in; each rated to 286 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 31.5 in, Width 45 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "15.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4130,7 +4130,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven polyester fabric upholstery in Ink, Blood Orange or Oyster, nailhead trim, dense foam padding, tapered wood legs, non-marking foot caps. Upholstered dining chair with a waisted hourglass back; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35.5 in, Width 25 in, Depth 23 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven polyester fabric upholstery in Ink, Blood Orange or Oyster, nailhead trim, dense foam padding, tapered wood legs, non-marking foot caps. Upholstered dining chair with a waisted hourglass back; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35.5 in, Width 25 in, Depth 23 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "20.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4152,7 +4152,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood frame in a choice of finishes, woven rattan seat in a natural tone. Café-style dining chair with a curved top rail, open crossed-splat back and tapered, splayed legs braced by curved hoops; 18.5 in seat height; arrives fully assembled; set of two chairs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.5 in, Width 39 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood frame in a choice of finishes, woven rattan seat in a natural tone. Café-style dining chair with a curved top rail, open crossed-splat back and tapered, splayed legs braced by curved hoops; 18.5 in seat height; arrives fully assembled; set of two chairs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.5 in, Width 39 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4174,7 +4174,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood frame in a choice of finishes with low stretchers between the legs, seat and back panel woven from natural twisted paper cord, plastic foot glides. Square-framed woven-seat dining side chair, also suited to use as an accent chair; rated to 330 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.5 in, Width 20 in, Depth 24 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood frame in a choice of finishes with low stretchers between the legs, seat and back panel woven from natural twisted paper cord, plastic foot glides. Square-framed woven-seat dining side chair, also suited to use as an accent chair; rated to 330 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34.5 in, Width 20 in, Depth 24 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "19 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4196,7 +4196,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven rattan cane seat and back, hardwood frame in Jet or Driftwood, rounded edges, ring stretcher, non-marking foot caps. Armless cane-back side chair for dining or as an accent chair; 18.5 in seat height; each rated to 330 lbs; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32 in, Width 17.5 in, Depth 20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven rattan cane seat and back, hardwood frame in Jet or Driftwood, rounded edges, ring stretcher, non-marking foot caps. Armless cane-back side chair for dining or as an accent chair; 18.5 in seat height; each rated to 330 lbs; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32 in, Width 17.5 in, Depth 20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "16 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4218,7 +4218,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven fabric upholstery in a choice of shades, dense foam padding in seat and back, deep button-tufted curved back, wooden legs in a dark finish, non-marking foot caps. Tall curved-back upholstered dining chair for the dining table, a home office desk, a hall or a living room; rated to 286 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 37.5 in, Width 18.5 in, Depth 24.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "21.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Woven fabric upholstery in a choice of shades, dense foam padding in seat and back, deep button-tufted curved back, wooden legs in a dark finish, non-marking foot caps. Tall curved-back upholstered dining chair for the dining table, a home office desk, a hall or a living room; rated to 286 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 37.5 in, Width 18.5 in, Depth 24.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "21.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4240,7 +4240,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Solid hardwood frame in Blonde or Chestnut finish, Tobacco or Jet vegan leather straps woven in a basket pattern for seat and back, crossbar stretchers, non-marking foot pads. Woven dining side chair with four straight legs; 17.5 in seat height for a standard dining table; each chair rated to 331 lbs; for dining rooms, living rooms, home offices and bedrooms; assembly required; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32.5 in, Width 20 in, Depth 22.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Solid hardwood frame in Blonde or Chestnut finish, Tobacco or Jet vegan leather straps woven in a basket pattern for seat and back, crossbar stretchers, non-marking foot pads. Woven dining side chair with four straight legs; 17.5 in seat height for a standard dining table; each chair rated to 331 lbs; for dining rooms, living rooms, home offices and bedrooms; assembly required; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32.5 in, Width 20 in, Depth 22.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4262,7 +4262,7 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in a warm wood finish, broad curved back board, thick dense foam padded seat, heathered weave fabric upholstery in Oyster or Cream, non-marking foot glides. Armless dining chairs, also suit a living room as accent chairs; set of two; rated to 551 lbs each; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.5 in, Width 17.1 in, Depth 21.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.095 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "15.55 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in a warm wood finish, broad curved back board, thick dense foam padded seat, heathered weave fabric upholstery in Oyster or Cream, non-marking foot glides. Armless dining chairs, also suit a living room as accent chairs; set of two; rated to 551 lbs each; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.5 in, Width 17.1 in, Depth 21.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.095 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "15.55 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4284,7 +4284,7 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Almond or Jet with curved backrest and sabre back legs, dense foam padded seat, heathered weave fabric upholstery in Cream, non-marking foot pins. Armless dining chairs for dining room, kitchen or as living room side chairs; set of two; rated to 330 lbs each; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.5 in, Width 20.5 in, Depth 21.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "2.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Almond or Jet with curved backrest and sabre back legs, dense foam padded seat, heathered weave fabric upholstery in Cream, non-marking foot pins. Armless dining chairs for dining room, kitchen or as living room side chairs; set of two; rated to 330 lbs each; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33.5 in, Width 20.5 in, Depth 21.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "2.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4306,7 +4306,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hard-wearing polyester fabric upholstery in Oyster or Dove, dense foam padding in seat and back, hardwood frame in Cocoa, curved framed back, tapered legs. Classic upholstered dining chairs, also accent chairs, set of two; rated to 500 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34 in, Width 23.5 in, Depth 22.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hard-wearing polyester fabric upholstery in Oyster or Dove, dense foam padding in seat and back, hardwood frame in Cocoa, curved framed back, tapered legs. Classic upholstered dining chairs, also accent chairs, set of two; rated to 500 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34 in, Width 23.5 in, Depth 22.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft bouclé upholstery in Cream or Dove spun from recycled plastic bottles, fabric certified to a recognised textile safety standard, hidden metal frame, padded curved backrest, splayed back legs, non-marking floor glides. Armless curved-back dining side chairs, also desk, guest or accent chairs, set of two; rated to 300 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 30.5 in, Width 19.5 in, Depth 23.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "2.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft bouclé upholstery in Cream or Dove spun from recycled plastic bottles, fabric certified to a recognised textile safety standard, hidden metal frame, padded curved backrest, splayed back legs, non-marking floor glides. Armless curved-back dining side chairs, also desk, guest or accent chairs, set of two; rated to 300 lbs."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 30.5 in, Width 19.5 in, Depth 23.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "2.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4350,7 +4350,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Chestnut, slub weave upholstery in Oyster or Charcoal, foam-padded seat cushion, removable back pillow, non-marking glides. Armless open-frame dining chair with tapered legs; doubles as an accent chair; rated to 300 lbs; comes fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 31 in, Width 20.5 in, Depth 22.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "21.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "2.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Chestnut, slub weave upholstery in Oyster or Charcoal, foam-padded seat cushion, removable back pillow, non-marking glides. Armless open-frame dining chair with tapered legs; doubles as an accent chair; rated to 300 lbs; comes fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 31 in, Width 20.5 in, Depth 22.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "21.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "2.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4372,7 +4372,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in Chambray or Pewter, dense foam padding, wood and plywood frame, splayed brushed Brass-tone stainless steel legs with non-marking caps, Brass-tone pull on the outer back for drawing the chair out. Scoop-back upholstered dining armchair with low sloping arms; also suits a desk, vanity, bedroom, living room or entryway; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34 in, Width 50 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in Chambray or Pewter, dense foam padding, wood and plywood frame, splayed brushed Brass-tone stainless steel legs with non-marking caps, Brass-tone pull on the outer back for drawing the chair out. Scoop-back upholstered dining armchair with low sloping arms; also suits a desk, vanity, bedroom, living room or entryway; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34 in, Width 50 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "19 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4394,7 +4394,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in Chambray or Charcoal, dense foam padding, wood and plywood frame, splayed brushed Brass-tone stainless steel legs with non-marking caps, Brass-tone pull on the outer back for drawing the chair out. Scoop-back upholstered dining armchair with low sloping arms; also suits a desk, vanity, bedroom, living room or entryway."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34 in, Width 25 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Stain-resistant performance velvet upholstery in Chambray or Charcoal, dense foam padding, wood and plywood frame, splayed brushed Brass-tone stainless steel legs with non-marking caps, Brass-tone pull on the outer back for drawing the chair out. Scoop-back upholstered dining armchair with low sloping arms; also suits a desk, vanity, bedroom, living room or entryway."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34 in, Width 25 in, Depth 22 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4416,7 +4416,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft chenille upholstery in Olive, Cream, Terracotta, Aegean or Truffle, dense foam padding, curved barrel back with enclosing arms, fully upholstered panel supports, non-marking floor glides. Rounded dining armchair that doubles as a bedroom or living room accent chair; seat height 19 in; rated to 330 lbs; no assembly needed."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 29.1 in, Width 23.4 in, Depth 23.6 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "25 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height above seat: ", "bold": true}, {"type": "text", "value": "6.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft chenille upholstery in Olive, Cream, Terracotta, Aegean or Truffle, dense foam padding, curved barrel back with enclosing arms, fully upholstered panel supports, non-marking floor glides. Rounded dining armchair that doubles as a bedroom or living room accent chair; seat height 19 in; rated to 330 lbs; no assembly needed."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 29.1 in, Width 23.4 in, Depth 23.6 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height: ", "bold": true}, {"type": "text", "value": "25 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Arm height above seat: ", "bold": true}, {"type": "text", "value": "6.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4438,7 +4438,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft textured chenille upholstery in Dove or Navy spun from recycled plastic bottles, fabric certified to a recognised textile safety standard, fully upholstered frame and legs, padded seat, non-marking floor glides. Armless upholstered dining side chair with a high square back, also a desk or accent chair; rated to 300 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32.5 in, Width 20.5 in, Depth 22.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "3 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Soft textured chenille upholstery in Dove or Navy spun from recycled plastic bottles, fabric certified to a recognised textile safety standard, fully upholstered frame and legs, padded seat, non-marking floor glides. Armless upholstered dining side chair with a high square back, also a desk or accent chair; rated to 300 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32.5 in, Width 20.5 in, Depth 22.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "3 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4460,7 +4460,7 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Textured slub-weave fabric upholstery in Oyster, Stone, Mink, Jet or Ink, dense foam padding, sturdy internal frame, non-marking floor glides. Armless slipper dining chair with a tall back and a waterfall seat front that folds down to the floor; 19.5 in seat height for a standard dining table; each chair rated to 300 lbs; suits dining rooms, vanities and living rooms; arrives fully assembled; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35.5 in, Width 19.5 in, Depth 24.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "3 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Textured slub-weave fabric upholstery in Oyster, Stone, Mink, Jet or Ink, dense foam padding, sturdy internal frame, non-marking floor glides. Armless slipper dining chair with a tall back and a waterfall seat front that folds down to the floor; 19.5 in seat height for a standard dining table; each chair rated to 300 lbs; suits dining rooms, vanities and living rooms; arrives fully assembled; set of two."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 35.5 in, Width 19.5 in, Depth 24.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Cushion thickness: ", "bold": true}, {"type": "text", "value": "3 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Honey or Jet, natural woven paper cord seat, curved back panel, X-shaped seat stretcher, non-marking floor glides. Armless dining side chair for kitchen or dining room; seat height about 18 in; rated to 497 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33 in, Width 19 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.9 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "15 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood frame in Honey or Jet, natural woven paper cord seat, curved back panel, X-shaped seat stretcher, non-marking floor glides. Armless dining side chair for kitchen or dining room; seat height about 18 in; rated to 497 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 33 in, Width 19 in, Depth 21 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat height: ", "bold": true}, {"type": "text", "value": "18.1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Seat depth: ", "bold": true}, {"type": "text", "value": "17.9 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "15 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4504,7 +4504,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood with wood-grain laminate in Almond, Jet or Chestnut, edge trim, tempered glass door windows, soft-close hinges, brass-tone ring pulls, wooden legs with felt pads. Tall arch-top display cabinet with an open arched shelf (rated 88 lbs), two glass-paned doors over two adjustable and one fixed shelf (70 lbs), and a closed lower compartment (84 lbs); for living rooms, halls and dining rooms; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 71 in, Width 31 in, Depth 17 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Shelf: ", "bold": true}, {"type": "text", "value": "Height 9 in, Width 27.5 in, Depth 13.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood with wood-grain laminate in Almond, Jet or Chestnut, edge trim, tempered glass door windows, soft-close hinges, brass-tone ring pulls, wooden legs with felt pads. Tall arch-top display cabinet with an open arched shelf (rated 88 lbs), two glass-paned doors over two adjustable and one fixed shelf (70 lbs), and a closed lower compartment (84 lbs); for living rooms, halls and dining rooms; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 71 in, Width 31 in, Depth 17 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Shelf: ", "bold": true}, {"type": "text", "value": "Height 9 in, Width 27.5 in, Depth 13.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4526,7 +4526,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood-grain finish in Oyster or Jet, open display shelving above, two soft-close lower doors with long vertical pulls over an adjustable shelf, rounded feet on non-marking glides. Tall arch-topped display cabinet and bookcase for living room, home office or dining room; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 78.7 in, Width 38 in, Depth 15.7 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Shelf: ", "bold": true}, {"type": "text", "value": "Height 13.5 in, Width 36.5 in, Depth 13.8 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood-grain finish in Oyster or Jet, open display shelving above, two soft-close lower doors with long vertical pulls over an adjustable shelf, rounded feet on non-marking glides. Tall arch-topped display cabinet and bookcase for living room, home office or dining room; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 78.7 in, Width 38 in, Depth 15.7 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Shelf: ", "bold": true}, {"type": "text", "value": "Height 13.5 in, Width 36.5 in, Depth 13.8 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4548,7 +4548,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood with wood-grain laminate finish in Jet or Almond, two push-to-open cupboards with raised grid panels, full-extension centre drawer, open media shelf with cable-management opening, tapered legs with central levelling legs. Low media cabinet that suits screens up to 65 in; rated to 198 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 22.8 in, Width 59.1 in, Depth 15.4 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "6.66 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Shelf: ", "bold": true}, {"type": "text", "value": "27.84 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood with wood-grain laminate finish in Jet or Almond, two push-to-open cupboards with raised grid panels, full-extension centre drawer, open media shelf with cable-management opening, tapered legs with central levelling legs. Low media cabinet that suits screens up to 65 in; rated to 198 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 22.8 in, Width 59.1 in, Depth 15.4 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "6.66 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Shelf: ", "bold": true}, {"type": "text", "value": "27.84 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4570,7 +4570,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood construction with a burl veneer in Chestnut or Cream, two drawers, two double-door cupboards with shelves, soft-close hinges, slim pulls, tapered legs, non-marking leveling feet. Sideboard, buffet, credenza or TV stand for screens up to 68 in; rated to 275 lbs; a TV set on top should be anchored; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34 in, Width 62 in, Depth 18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood construction with a burl veneer in Chestnut or Cream, two drawers, two double-door cupboards with shelves, soft-close hinges, slim pulls, tapered legs, non-marking leveling feet. Sideboard, buffet, credenza or TV stand for screens up to 68 in; rated to 275 lbs; a TV set on top should be anchored; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 34 in, Width 62 in, Depth 18 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4592,7 +4592,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood frame with a laminate wood-grain surface in Hazel or Almond, four slatted doors with press-to-open latches and soft-close hinges, adjustable interior shelves, four cable holes for cord management, recessed plinth base. Long, low four-door sideboard for dining storage, credenza use or as a media cabinet beneath a wall-mounted or securely anchored television; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 29.7 in, Width 70.8 in, Depth 16.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside: ", "bold": true}, {"type": "text", "value": "2.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Height 25.8 in, Width 34 in, Depth 16 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood frame with a laminate wood-grain surface in Hazel or Almond, four slatted doors with press-to-open latches and soft-close hinges, adjustable interior shelves, four cable holes for cord management, recessed plinth base. Long, low four-door sideboard for dining storage, credenza use or as a media cabinet beneath a wall-mounted or securely anchored television; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 29.7 in, Width 70.8 in, Depth 16.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside: ", "bold": true}, {"type": "text", "value": "2.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Height 25.8 in, Width 34 in, Depth 16 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4614,7 +4614,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood with a wood-grain veneer finish in Almond or Cocoa, woven paper cord open lower shelf, four doors, fixed interior shelf, slim metal pulls, rounded corner legs. Long low sideboard for dining room, living room, entry or office; only the doors attach on arrival; weight capacity not stated."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32 in, Width 68 in, Depth 18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Height 17.8 in, Width 28.1 in, Depth 14.3 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood with a wood-grain veneer finish in Almond or Cocoa, woven paper cord open lower shelf, four doors, fixed interior shelf, slim metal pulls, rounded corner legs. Long low sideboard for dining room, living room, entry or office; only the doors attach on arrival; weight capacity not stated."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32 in, Width 68 in, Depth 18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Clearance between legs: ", "bold": true}, {"type": "text", "value": "Height 17.8 in, Width 28.1 in, Depth 14.3 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4636,7 +4636,7 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Sturdy engineered wood finished in Almond, Hazel or White. Three-piece home office set: a leaning, tiered ladder-frame desk with a work surface, three shelves above it and a pair of pull-out drawers, plus two narrow bookcases, each with three open shelves over a single-door cupboard for concealed storage."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 71 in, Width 90 in, Depth 18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "4.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "0.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Sturdy engineered wood finished in Almond, Hazel or White. Three-piece home office set: a leaning, tiered ladder-frame desk with a work surface, three shelves above it and a pair of pull-out drawers, plus two narrow bookcases, each with three open shelves over a single-door cupboard for concealed storage."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 71 in, Width 90 in, Depth 18.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "4.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "0.5 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4658,7 +4658,7 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood frame and four open wood shelves in Blonde, Jet or Chestnut, matching arched frames front and back, open back and sides, non-marking glides. Mid-height open bookcase, 5 ft high, for books, collected pieces and display; shelves hold up to 220 lbs in all; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 60 in, Width 30 in, Depth 14.1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Shelf: ", "bold": true}, {"type": "text", "value": "Height 1.2 in, Width 30 in, Depth 14.1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood frame and four open wood shelves in Blonde, Jet or Chestnut, matching arched frames front and back, open back and sides, non-marking glides. Mid-height open bookcase, 5 ft high, for books, collected pieces and display; shelves hold up to 220 lbs in all; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 60 in, Width 30 in, Depth 14.1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Shelf: ", "bold": true}, {"type": "text", "value": "Height 1.2 in, Width 30 in, Depth 14.1 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4680,7 +4680,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Steel tube frame in Chrome or Jet, tempered glass top, telescoping upright with five height settings, open C-shaped base that slides under a sofa or bed, non-marking foot caps. Round adjustable side table for drinks, trays, laptops or plants; rated to 17 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 37.5 in, Width 20 in, Depth 20 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Steel tube frame in Chrome or Jet, tempered glass top, telescoping upright with five height settings, open C-shaped base that slides under a sofa or bed, non-marking foot caps. Round adjustable side table for drinks, trays, laptops or plants; rated to 17 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 37.5 in, Width 20 in, Depth 20 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4702,7 +4702,7 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Natural marble column base, iron rod and round iron top in a White, Jet or Brass finish, non-marking pad. Slim side table for beside a sofa, hall armchair or reading chair; rated to 99 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20 in, Width 14 in, Depth 14 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Natural marble column base, iron rod and round iron top in a White, Jet or Brass finish, non-marking pad. Slim side table for beside a sofa, hall armchair or reading chair; rated to 99 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20 in, Width 14 in, Depth 14 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4724,7 +4724,7 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood top in Hazel, iron pedestal column and round disc base in a Brass or Jet finish, non-marking floor pad. Round pedestal side table for living room, bedroom, hallway or entryway; rated to 100 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 19.5 in, Width 19.5 in, Depth 19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Wood top in Hazel, iron pedestal column and round disc base in a Brass or Jet finish, non-marking floor pad. Round pedestal side table for living room, bedroom, hallway or entryway; rated to 100 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 19.5 in, Width 19.5 in, Depth 19.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "19 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "1 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4746,7 +4746,7 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood in Chestnut or Jet, felt floor pads. Round side table with a thick, softly rounded top on three tall cylindrical legs; end table, bedside table or plant stand; rated to 200 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20.5 in, Width 18 in, Depth 18 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood in Chestnut or Jet, felt floor pads. Round side table with a thick, softly rounded top on three tall cylindrical legs; end table, bedside table or plant stand; rated to 200 lbs; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20.5 in, Width 18 in, Depth 18 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4768,7 +4768,7 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood with a wood-grain laminate finish in Jet or Almond, woven rattan drawer fronts, two drawers on full-extension glides, metal knobs, open lower shelf, straight legs on non-marking feet. Slim console table for entry, hallway or as a TV console; rated to 132 lbs on top and 132 lbs on the shelf; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32 in, Width 46.5 in, Depth 14 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "24 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Engineered wood with a wood-grain laminate finish in Jet or Almond, woven rattan drawer fronts, two drawers on full-extension glides, metal knobs, open lower shelf, straight legs on non-marking feet. Slim console table for entry, hallway or as a TV console; rated to 132 lbs on top and 132 lbs on the shelf; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32 in, Width 46.5 in, Depth 14 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Floor to underside of top: ", "bold": true}, {"type": "text", "value": "24 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4790,7 +4790,7 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood in Chestnut or Almond, adjustable non-marking feet for levelling on uneven floors. Low rectangular coffee table with a board top and two broad split-panel legs, rounded edges; room for several mugs, books and a tray; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 16.5 in, Width 44 in, Depth 26 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "1 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Hardwood in Chestnut or Almond, adjustable non-marking feet for levelling on uneven floors. Low rectangular coffee table with a board top and two broad split-panel legs, rounded edges; room for several mugs, books and a tray; assembly required."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 16.5 in, Width 44 in, Depth 26 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Tabletop thickness: ", "bold": true}, {"type": "text", "value": "1 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4812,7 +4812,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood in Jet or Chestnut. Round side table with a raised-lip tray top on a solid bell-shaped pedestal; end table, bedside table or plant stand; rated to 200 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20.5 in, Width 15 in, Depth 15 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "100% solid hardwood in Jet or Chestnut. Round side table with a raised-lip tray top on a solid bell-shaped pedestal; end table, bedside table or plant stand; rated to 200 lbs; arrives fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 20.5 in, Width 15 in, Depth 15 in"}]}]}</t>
         </is>
       </c>
     </row>
@@ -4966,7 +4966,7 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Premium fabric slipcover upholstery (ticking stripe, windowpane check or plain weave, depending on colour), dense foam padding, protective foot pins. Curved/rounded shelter-arm back silhouette, slipcovered form, includes accent pillow, fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32.5 in, Width 29 in, Depth 32.5 in"}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Weight: ", "bold": true}, {"type": "text", "value": "TBD."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Boxed dimensions: ", "bold": true}, {"type": "text", "value": "TBD."}]}]}</t>
+          <t>{"type": "root", "children": [{"type": "paragraph", "children": [{"type": "text", "value": "Materials: ", "bold": true}, {"type": "text", "value": "Premium fabric slipcover upholstery (ticking stripe, windowpane check or plain weave, depending on colour), dense foam padding, protective foot pins. Curved/rounded shelter-arm back silhouette, slipcovered form, includes accent pillow, fully assembled."}]}, {"type": "paragraph", "children": [{"type": "text", "value": "Product dimensions: ", "bold": true}, {"type": "text", "value": "Height 32.5 in, Width 29 in, Depth 32.5 in"}]}]}</t>
         </is>
       </c>
     </row>

</xml_diff>